<commit_message>
antes de implementar la encriptacion
antes de implementar la encriptacion
</commit_message>
<xml_diff>
--- a/evaluaciones-frontend/public/assets/formato_banco_preguntas_asig_EF.xlsx
+++ b/evaluaciones-frontend/public/assets/formato_banco_preguntas_asig_EF.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALIDACIONES" sheetId="1" r:id="Rbba302b41ad0488e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R4ffcd0418cce4019"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banco" sheetId="3" r:id="Rb1380b0a6c2d4a88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplo" sheetId="4" r:id="R1309618bc3bd4e84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALIDACIONES" sheetId="1" r:id="R1432f8ed1b7f4b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R2aab5973f6ab462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banco" sheetId="3" r:id="Rb0b3f63805c24dbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplo" sheetId="4" r:id="R3eae356e06d54c37"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="LISTA_TIPOS_2P">VALIDACIONES!$A$1:$A$8</x:definedName>
@@ -253,9 +253,6 @@
     <x:t xml:space="preserve">parcial</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">observaciones</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">_obs_1</x:t>
   </x:si>
   <x:si>
@@ -268,43 +265,7 @@
     <x:t xml:space="preserve">_obs_4</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Grupo 1 (VF simple + complejas + A/B):</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Grupo 2 (Mejor respuesta):</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Grupo 3 (Casos/problemas y emp.):</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NOTAS DE CARGA</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1. La columna L te dira si la fila esta OK o que campos faltan/revisar.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">2. Casos/problemas y Emparejamiento Ampliado usan grupo y enunciado, pero no respuesta_correcta ni dificultad.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">3. Emparejamiento Ampliado puede usar de 2 a 5 claves en opcion_a a opcion_e.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">4. En Verdadero o Falso Simple, opcion_a, opcion_b y respuesta_correcta se preparan automaticamente.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">5. En Respuesta A/B/Ambas/Ninguna, escriba solo I. y II. en el enunciado; opcion_a a opcion_d se preparan con: A. Si la primera es verdadera | B. Si la segunda es verdadera | C. Si ambas son verdaderas | D. Si ninguna es verdadera.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">6. En Verdadero o Falso Complejas, escriba 1. a 4. en opcion_a a opcion_d; opcion_e queda deshabilitada.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">7. En Emparejamiento Ampliado, el enunciado se prepara con: De la lista de opciones, seleccione la respuesta correcta para cada enunciado</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">8. Este formato esta preparado para EF (Examen Final).</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">9. Los grupos de conteo por tipo no consideran casos/problemas ni emparejamientos porque funcionan como cabeceras.</x:t>
+    <x:t xml:space="preserve">observaciones</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">El agua hierve a 100 grados Celsius al nivel del mar.</x:t>
@@ -527,7 +488,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -562,6 +523,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF006064"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3EEFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -624,7 +590,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -710,6 +676,24 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1417,7 +1401,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
-        <x:v>imagen_base64</x:v>
+        <x:v>M (imagen_base64)</x:v>
       </x:c>
       <x:c r="B27" t="str">
         <x:v>Imagen opcional. Puede incluir #sea-size=GRANDE, MEDIANA, PEQUENA o MUY_PEQUENA; MEDIANA es el tamaño predeterminado.</x:v>
@@ -1473,12 +1457,36 @@
     <x:col min="4" max="8" width="25" style="6" customWidth="1"/>
     <x:col min="9" max="9" width="20" customWidth="1"/>
     <x:col min="10" max="11" width="12" customWidth="1"/>
-    <x:col min="12" max="12" width="34" style="6" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="28" style="6" hidden="0" customWidth="1"/>
     <x:col min="13" max="36" width="3" hidden="1" customWidth="1"/>
-    <x:col min="13" max="13" width="28" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="34" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="3" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="11" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="36" max="36" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="37" max="37" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="38" max="38" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="39" max="39" width="0.10000000149011612" hidden="0" customWidth="1"/>
+    <x:col min="40" max="40" width="0.10000000149011612" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1516,85 +1524,85 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="L1" s="7" t="str">
+        <x:v>observaciones</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
         <x:v>imagen_base64</x:v>
-      </x:c>
-      <x:c r="M1" t="s">
-        <x:v>74</x:v>
       </x:c>
       <x:c r="N1"/>
       <x:c r="O1"/>
       <x:c r="P1"/>
       <x:c r="Q1" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="R1" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="R1" t="s">
+      <x:c r="S1" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="S1" t="s">
+      <x:c r="T1" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="T1" t="s">
-        <x:v>78</x:v>
-      </x:c>
       <x:c r="U1" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="V1" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="V1" t="s">
+      <x:c r="W1" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="W1" t="s">
+      <x:c r="X1" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="X1" t="s">
-        <x:v>78</x:v>
-      </x:c>
       <x:c r="Y1" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="Z1" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="Z1" t="s">
+      <x:c r="AA1" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="AA1" t="s">
+      <x:c r="AB1" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="AB1" t="s">
-        <x:v>78</x:v>
-      </x:c>
       <x:c r="AC1" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="AD1" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="AD1" t="s">
+      <x:c r="AE1" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="AE1" t="s">
+      <x:c r="AF1" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="AF1" t="s">
-        <x:v>78</x:v>
-      </x:c>
       <x:c r="AG1" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="AH1" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="AH1" t="s">
+      <x:c r="AI1" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="AI1" t="s">
+      <x:c r="AJ1" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="AJ1" t="s">
-        <x:v>78</x:v>
-      </x:c>
       <x:c r="AK1" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="AL1" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="AL1" t="s">
+      <x:c r="AM1" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="AM1" t="s">
+      <x:c r="AN1" t="s">
         <x:v>77</x:v>
-      </x:c>
-      <x:c r="AN1" t="s">
-        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
@@ -1631,11 +1639,11 @@
       <x:c r="K2" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L2" s="10"/>
-      <x:c r="M2" t="str">
+      <x:c r="L2" s="10" t="str">
         <x:f>IF(TRIM($A2)="","",IF(COUNTIF($Q2:$AK2,"?*")=0,"OK","Falta revisar: "&amp;$Q2&amp;$R2&amp;$S2&amp;$T2&amp;$U2&amp;$V2&amp;$W2&amp;$X2&amp;$Y2&amp;$Z2&amp;$AA2&amp;$AB2&amp;$AC2&amp;$AD2&amp;$AE2&amp;$AF2&amp;$AG2&amp;$AH2&amp;$AI2&amp;$AJ2&amp;$AK2))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M2"/>
       <x:c r="N2"/>
       <x:c r="O2"/>
       <x:c r="P2"/>
@@ -1747,11 +1755,11 @@
       <x:c r="K3" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L3" s="10"/>
-      <x:c r="M3" t="str">
+      <x:c r="L3" s="10" t="str">
         <x:f>IF(TRIM($A3)="","",IF(COUNTIF($Q3:$AK3,"?*")=0,"OK","Falta revisar: "&amp;$Q3&amp;$R3&amp;$S3&amp;$T3&amp;$U3&amp;$V3&amp;$W3&amp;$X3&amp;$Y3&amp;$Z3&amp;$AA3&amp;$AB3&amp;$AC3&amp;$AD3&amp;$AE3&amp;$AF3&amp;$AG3&amp;$AH3&amp;$AI3&amp;$AJ3&amp;$AK3))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M3"/>
       <x:c r="N3"/>
       <x:c r="O3"/>
       <x:c r="P3"/>
@@ -1863,11 +1871,11 @@
       <x:c r="K4" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L4" s="10"/>
-      <x:c r="M4" t="str">
+      <x:c r="L4" s="10" t="str">
         <x:f>IF(TRIM($A4)="","",IF(COUNTIF($Q4:$AK4,"?*")=0,"OK","Falta revisar: "&amp;$Q4&amp;$R4&amp;$S4&amp;$T4&amp;$U4&amp;$V4&amp;$W4&amp;$X4&amp;$Y4&amp;$Z4&amp;$AA4&amp;$AB4&amp;$AC4&amp;$AD4&amp;$AE4&amp;$AF4&amp;$AG4&amp;$AH4&amp;$AI4&amp;$AJ4&amp;$AK4))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M4"/>
       <x:c r="N4"/>
       <x:c r="O4"/>
       <x:c r="P4"/>
@@ -1979,11 +1987,11 @@
       <x:c r="K5" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L5" s="10"/>
-      <x:c r="M5" t="str">
+      <x:c r="L5" s="10" t="str">
         <x:f>IF(TRIM($A5)="","",IF(COUNTIF($Q5:$AK5,"?*")=0,"OK","Falta revisar: "&amp;$Q5&amp;$R5&amp;$S5&amp;$T5&amp;$U5&amp;$V5&amp;$W5&amp;$X5&amp;$Y5&amp;$Z5&amp;$AA5&amp;$AB5&amp;$AC5&amp;$AD5&amp;$AE5&amp;$AF5&amp;$AG5&amp;$AH5&amp;$AI5&amp;$AJ5&amp;$AK5))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M5"/>
       <x:c r="N5"/>
       <x:c r="O5"/>
       <x:c r="P5"/>
@@ -2095,11 +2103,11 @@
       <x:c r="K6" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L6" s="10"/>
-      <x:c r="M6" t="str">
+      <x:c r="L6" s="10" t="str">
         <x:f>IF(TRIM($A6)="","",IF(COUNTIF($Q6:$AK6,"?*")=0,"OK","Falta revisar: "&amp;$Q6&amp;$R6&amp;$S6&amp;$T6&amp;$U6&amp;$V6&amp;$W6&amp;$X6&amp;$Y6&amp;$Z6&amp;$AA6&amp;$AB6&amp;$AC6&amp;$AD6&amp;$AE6&amp;$AF6&amp;$AG6&amp;$AH6&amp;$AI6&amp;$AJ6&amp;$AK6))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M6"/>
       <x:c r="N6"/>
       <x:c r="O6"/>
       <x:c r="P6"/>
@@ -2211,11 +2219,11 @@
       <x:c r="K7" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L7" s="10"/>
-      <x:c r="M7" t="str">
+      <x:c r="L7" s="10" t="str">
         <x:f>IF(TRIM($A7)="","",IF(COUNTIF($Q7:$AK7,"?*")=0,"OK","Falta revisar: "&amp;$Q7&amp;$R7&amp;$S7&amp;$T7&amp;$U7&amp;$V7&amp;$W7&amp;$X7&amp;$Y7&amp;$Z7&amp;$AA7&amp;$AB7&amp;$AC7&amp;$AD7&amp;$AE7&amp;$AF7&amp;$AG7&amp;$AH7&amp;$AI7&amp;$AJ7&amp;$AK7))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M7"/>
       <x:c r="N7"/>
       <x:c r="O7"/>
       <x:c r="P7"/>
@@ -2327,11 +2335,11 @@
       <x:c r="K8" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L8" s="10"/>
-      <x:c r="M8" t="str">
+      <x:c r="L8" s="10" t="str">
         <x:f>IF(TRIM($A8)="","",IF(COUNTIF($Q8:$AK8,"?*")=0,"OK","Falta revisar: "&amp;$Q8&amp;$R8&amp;$S8&amp;$T8&amp;$U8&amp;$V8&amp;$W8&amp;$X8&amp;$Y8&amp;$Z8&amp;$AA8&amp;$AB8&amp;$AC8&amp;$AD8&amp;$AE8&amp;$AF8&amp;$AG8&amp;$AH8&amp;$AI8&amp;$AJ8&amp;$AK8))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M8"/>
       <x:c r="N8"/>
       <x:c r="O8"/>
       <x:c r="P8"/>
@@ -2443,11 +2451,11 @@
       <x:c r="K9" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L9" s="10"/>
-      <x:c r="M9" t="str">
+      <x:c r="L9" s="10" t="str">
         <x:f>IF(TRIM($A9)="","",IF(COUNTIF($Q9:$AK9,"?*")=0,"OK","Falta revisar: "&amp;$Q9&amp;$R9&amp;$S9&amp;$T9&amp;$U9&amp;$V9&amp;$W9&amp;$X9&amp;$Y9&amp;$Z9&amp;$AA9&amp;$AB9&amp;$AC9&amp;$AD9&amp;$AE9&amp;$AF9&amp;$AG9&amp;$AH9&amp;$AI9&amp;$AJ9&amp;$AK9))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M9"/>
       <x:c r="N9"/>
       <x:c r="O9"/>
       <x:c r="P9"/>
@@ -2559,11 +2567,11 @@
       <x:c r="K10" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L10" s="10"/>
-      <x:c r="M10" t="str">
+      <x:c r="L10" s="10" t="str">
         <x:f>IF(TRIM($A10)="","",IF(COUNTIF($Q10:$AK10,"?*")=0,"OK","Falta revisar: "&amp;$Q10&amp;$R10&amp;$S10&amp;$T10&amp;$U10&amp;$V10&amp;$W10&amp;$X10&amp;$Y10&amp;$Z10&amp;$AA10&amp;$AB10&amp;$AC10&amp;$AD10&amp;$AE10&amp;$AF10&amp;$AG10&amp;$AH10&amp;$AI10&amp;$AJ10&amp;$AK10))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M10"/>
       <x:c r="N10"/>
       <x:c r="O10"/>
       <x:c r="P10"/>
@@ -2675,11 +2683,11 @@
       <x:c r="K11" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L11" s="10"/>
-      <x:c r="M11" t="str">
+      <x:c r="L11" s="10" t="str">
         <x:f>IF(TRIM($A11)="","",IF(COUNTIF($Q11:$AK11,"?*")=0,"OK","Falta revisar: "&amp;$Q11&amp;$R11&amp;$S11&amp;$T11&amp;$U11&amp;$V11&amp;$W11&amp;$X11&amp;$Y11&amp;$Z11&amp;$AA11&amp;$AB11&amp;$AC11&amp;$AD11&amp;$AE11&amp;$AF11&amp;$AG11&amp;$AH11&amp;$AI11&amp;$AJ11&amp;$AK11))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M11"/>
       <x:c r="N11"/>
       <x:c r="O11"/>
       <x:c r="P11"/>
@@ -2791,11 +2799,11 @@
       <x:c r="K12" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L12" s="10"/>
-      <x:c r="M12" t="str">
+      <x:c r="L12" s="10" t="str">
         <x:f>IF(TRIM($A12)="","",IF(COUNTIF($Q12:$AK12,"?*")=0,"OK","Falta revisar: "&amp;$Q12&amp;$R12&amp;$S12&amp;$T12&amp;$U12&amp;$V12&amp;$W12&amp;$X12&amp;$Y12&amp;$Z12&amp;$AA12&amp;$AB12&amp;$AC12&amp;$AD12&amp;$AE12&amp;$AF12&amp;$AG12&amp;$AH12&amp;$AI12&amp;$AJ12&amp;$AK12))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M12"/>
       <x:c r="N12"/>
       <x:c r="O12"/>
       <x:c r="P12"/>
@@ -2907,11 +2915,11 @@
       <x:c r="K13" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L13" s="10"/>
-      <x:c r="M13" t="str">
+      <x:c r="L13" s="10" t="str">
         <x:f>IF(TRIM($A13)="","",IF(COUNTIF($Q13:$AK13,"?*")=0,"OK","Falta revisar: "&amp;$Q13&amp;$R13&amp;$S13&amp;$T13&amp;$U13&amp;$V13&amp;$W13&amp;$X13&amp;$Y13&amp;$Z13&amp;$AA13&amp;$AB13&amp;$AC13&amp;$AD13&amp;$AE13&amp;$AF13&amp;$AG13&amp;$AH13&amp;$AI13&amp;$AJ13&amp;$AK13))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M13"/>
       <x:c r="N13"/>
       <x:c r="O13"/>
       <x:c r="P13"/>
@@ -3023,11 +3031,11 @@
       <x:c r="K14" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L14" s="10"/>
-      <x:c r="M14" t="str">
+      <x:c r="L14" s="10" t="str">
         <x:f>IF(TRIM($A14)="","",IF(COUNTIF($Q14:$AK14,"?*")=0,"OK","Falta revisar: "&amp;$Q14&amp;$R14&amp;$S14&amp;$T14&amp;$U14&amp;$V14&amp;$W14&amp;$X14&amp;$Y14&amp;$Z14&amp;$AA14&amp;$AB14&amp;$AC14&amp;$AD14&amp;$AE14&amp;$AF14&amp;$AG14&amp;$AH14&amp;$AI14&amp;$AJ14&amp;$AK14))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M14"/>
       <x:c r="N14"/>
       <x:c r="O14"/>
       <x:c r="P14"/>
@@ -3139,11 +3147,11 @@
       <x:c r="K15" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L15" s="10"/>
-      <x:c r="M15" t="str">
+      <x:c r="L15" s="10" t="str">
         <x:f>IF(TRIM($A15)="","",IF(COUNTIF($Q15:$AK15,"?*")=0,"OK","Falta revisar: "&amp;$Q15&amp;$R15&amp;$S15&amp;$T15&amp;$U15&amp;$V15&amp;$W15&amp;$X15&amp;$Y15&amp;$Z15&amp;$AA15&amp;$AB15&amp;$AC15&amp;$AD15&amp;$AE15&amp;$AF15&amp;$AG15&amp;$AH15&amp;$AI15&amp;$AJ15&amp;$AK15))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M15"/>
       <x:c r="N15"/>
       <x:c r="O15"/>
       <x:c r="P15"/>
@@ -3255,11 +3263,11 @@
       <x:c r="K16" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L16" s="10"/>
-      <x:c r="M16" t="str">
+      <x:c r="L16" s="10" t="str">
         <x:f>IF(TRIM($A16)="","",IF(COUNTIF($Q16:$AK16,"?*")=0,"OK","Falta revisar: "&amp;$Q16&amp;$R16&amp;$S16&amp;$T16&amp;$U16&amp;$V16&amp;$W16&amp;$X16&amp;$Y16&amp;$Z16&amp;$AA16&amp;$AB16&amp;$AC16&amp;$AD16&amp;$AE16&amp;$AF16&amp;$AG16&amp;$AH16&amp;$AI16&amp;$AJ16&amp;$AK16))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M16"/>
       <x:c r="N16"/>
       <x:c r="O16"/>
       <x:c r="P16"/>
@@ -3371,11 +3379,11 @@
       <x:c r="K17" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L17" s="10"/>
-      <x:c r="M17" t="str">
+      <x:c r="L17" s="10" t="str">
         <x:f>IF(TRIM($A17)="","",IF(COUNTIF($Q17:$AK17,"?*")=0,"OK","Falta revisar: "&amp;$Q17&amp;$R17&amp;$S17&amp;$T17&amp;$U17&amp;$V17&amp;$W17&amp;$X17&amp;$Y17&amp;$Z17&amp;$AA17&amp;$AB17&amp;$AC17&amp;$AD17&amp;$AE17&amp;$AF17&amp;$AG17&amp;$AH17&amp;$AI17&amp;$AJ17&amp;$AK17))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M17"/>
       <x:c r="N17"/>
       <x:c r="O17"/>
       <x:c r="P17"/>
@@ -3487,11 +3495,11 @@
       <x:c r="K18" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L18" s="10"/>
-      <x:c r="M18" t="str">
+      <x:c r="L18" s="10" t="str">
         <x:f>IF(TRIM($A18)="","",IF(COUNTIF($Q18:$AK18,"?*")=0,"OK","Falta revisar: "&amp;$Q18&amp;$R18&amp;$S18&amp;$T18&amp;$U18&amp;$V18&amp;$W18&amp;$X18&amp;$Y18&amp;$Z18&amp;$AA18&amp;$AB18&amp;$AC18&amp;$AD18&amp;$AE18&amp;$AF18&amp;$AG18&amp;$AH18&amp;$AI18&amp;$AJ18&amp;$AK18))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M18"/>
       <x:c r="N18"/>
       <x:c r="O18"/>
       <x:c r="P18"/>
@@ -3603,11 +3611,11 @@
       <x:c r="K19" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L19" s="10"/>
-      <x:c r="M19" t="str">
+      <x:c r="L19" s="10" t="str">
         <x:f>IF(TRIM($A19)="","",IF(COUNTIF($Q19:$AK19,"?*")=0,"OK","Falta revisar: "&amp;$Q19&amp;$R19&amp;$S19&amp;$T19&amp;$U19&amp;$V19&amp;$W19&amp;$X19&amp;$Y19&amp;$Z19&amp;$AA19&amp;$AB19&amp;$AC19&amp;$AD19&amp;$AE19&amp;$AF19&amp;$AG19&amp;$AH19&amp;$AI19&amp;$AJ19&amp;$AK19))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M19"/>
       <x:c r="N19"/>
       <x:c r="O19"/>
       <x:c r="P19"/>
@@ -3719,11 +3727,11 @@
       <x:c r="K20" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L20" s="10"/>
-      <x:c r="M20" t="str">
+      <x:c r="L20" s="10" t="str">
         <x:f>IF(TRIM($A20)="","",IF(COUNTIF($Q20:$AK20,"?*")=0,"OK","Falta revisar: "&amp;$Q20&amp;$R20&amp;$S20&amp;$T20&amp;$U20&amp;$V20&amp;$W20&amp;$X20&amp;$Y20&amp;$Z20&amp;$AA20&amp;$AB20&amp;$AC20&amp;$AD20&amp;$AE20&amp;$AF20&amp;$AG20&amp;$AH20&amp;$AI20&amp;$AJ20&amp;$AK20))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M20"/>
       <x:c r="N20"/>
       <x:c r="O20"/>
       <x:c r="P20"/>
@@ -3835,11 +3843,11 @@
       <x:c r="K21" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L21" s="10"/>
-      <x:c r="M21" t="str">
+      <x:c r="L21" s="10" t="str">
         <x:f>IF(TRIM($A21)="","",IF(COUNTIF($Q21:$AK21,"?*")=0,"OK","Falta revisar: "&amp;$Q21&amp;$R21&amp;$S21&amp;$T21&amp;$U21&amp;$V21&amp;$W21&amp;$X21&amp;$Y21&amp;$Z21&amp;$AA21&amp;$AB21&amp;$AC21&amp;$AD21&amp;$AE21&amp;$AF21&amp;$AG21&amp;$AH21&amp;$AI21&amp;$AJ21&amp;$AK21))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M21"/>
       <x:c r="N21"/>
       <x:c r="O21"/>
       <x:c r="P21"/>
@@ -3951,11 +3959,11 @@
       <x:c r="K22" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L22" s="10"/>
-      <x:c r="M22" t="str">
+      <x:c r="L22" s="10" t="str">
         <x:f>IF(TRIM($A22)="","",IF(COUNTIF($Q22:$AK22,"?*")=0,"OK","Falta revisar: "&amp;$Q22&amp;$R22&amp;$S22&amp;$T22&amp;$U22&amp;$V22&amp;$W22&amp;$X22&amp;$Y22&amp;$Z22&amp;$AA22&amp;$AB22&amp;$AC22&amp;$AD22&amp;$AE22&amp;$AF22&amp;$AG22&amp;$AH22&amp;$AI22&amp;$AJ22&amp;$AK22))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M22"/>
       <x:c r="N22"/>
       <x:c r="O22"/>
       <x:c r="P22"/>
@@ -4067,11 +4075,11 @@
       <x:c r="K23" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L23" s="10"/>
-      <x:c r="M23" t="str">
+      <x:c r="L23" s="10" t="str">
         <x:f>IF(TRIM($A23)="","",IF(COUNTIF($Q23:$AK23,"?*")=0,"OK","Falta revisar: "&amp;$Q23&amp;$R23&amp;$S23&amp;$T23&amp;$U23&amp;$V23&amp;$W23&amp;$X23&amp;$Y23&amp;$Z23&amp;$AA23&amp;$AB23&amp;$AC23&amp;$AD23&amp;$AE23&amp;$AF23&amp;$AG23&amp;$AH23&amp;$AI23&amp;$AJ23&amp;$AK23))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M23"/>
       <x:c r="N23"/>
       <x:c r="O23"/>
       <x:c r="P23"/>
@@ -4183,11 +4191,11 @@
       <x:c r="K24" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L24" s="10"/>
-      <x:c r="M24" t="str">
+      <x:c r="L24" s="10" t="str">
         <x:f>IF(TRIM($A24)="","",IF(COUNTIF($Q24:$AK24,"?*")=0,"OK","Falta revisar: "&amp;$Q24&amp;$R24&amp;$S24&amp;$T24&amp;$U24&amp;$V24&amp;$W24&amp;$X24&amp;$Y24&amp;$Z24&amp;$AA24&amp;$AB24&amp;$AC24&amp;$AD24&amp;$AE24&amp;$AF24&amp;$AG24&amp;$AH24&amp;$AI24&amp;$AJ24&amp;$AK24))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M24"/>
       <x:c r="N24"/>
       <x:c r="O24"/>
       <x:c r="P24"/>
@@ -4299,11 +4307,11 @@
       <x:c r="K25" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L25" s="10"/>
-      <x:c r="M25" t="str">
+      <x:c r="L25" s="10" t="str">
         <x:f>IF(TRIM($A25)="","",IF(COUNTIF($Q25:$AK25,"?*")=0,"OK","Falta revisar: "&amp;$Q25&amp;$R25&amp;$S25&amp;$T25&amp;$U25&amp;$V25&amp;$W25&amp;$X25&amp;$Y25&amp;$Z25&amp;$AA25&amp;$AB25&amp;$AC25&amp;$AD25&amp;$AE25&amp;$AF25&amp;$AG25&amp;$AH25&amp;$AI25&amp;$AJ25&amp;$AK25))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M25"/>
       <x:c r="N25"/>
       <x:c r="O25"/>
       <x:c r="P25"/>
@@ -4415,11 +4423,11 @@
       <x:c r="K26" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L26" s="10"/>
-      <x:c r="M26" t="str">
+      <x:c r="L26" s="10" t="str">
         <x:f>IF(TRIM($A26)="","",IF(COUNTIF($Q26:$AK26,"?*")=0,"OK","Falta revisar: "&amp;$Q26&amp;$R26&amp;$S26&amp;$T26&amp;$U26&amp;$V26&amp;$W26&amp;$X26&amp;$Y26&amp;$Z26&amp;$AA26&amp;$AB26&amp;$AC26&amp;$AD26&amp;$AE26&amp;$AF26&amp;$AG26&amp;$AH26&amp;$AI26&amp;$AJ26&amp;$AK26))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M26"/>
       <x:c r="N26"/>
       <x:c r="O26"/>
       <x:c r="P26"/>
@@ -4531,11 +4539,11 @@
       <x:c r="K27" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L27" s="10"/>
-      <x:c r="M27" t="str">
+      <x:c r="L27" s="10" t="str">
         <x:f>IF(TRIM($A27)="","",IF(COUNTIF($Q27:$AK27,"?*")=0,"OK","Falta revisar: "&amp;$Q27&amp;$R27&amp;$S27&amp;$T27&amp;$U27&amp;$V27&amp;$W27&amp;$X27&amp;$Y27&amp;$Z27&amp;$AA27&amp;$AB27&amp;$AC27&amp;$AD27&amp;$AE27&amp;$AF27&amp;$AG27&amp;$AH27&amp;$AI27&amp;$AJ27&amp;$AK27))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M27"/>
       <x:c r="N27"/>
       <x:c r="O27"/>
       <x:c r="P27"/>
@@ -4647,11 +4655,11 @@
       <x:c r="K28" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L28" s="10"/>
-      <x:c r="M28" t="str">
+      <x:c r="L28" s="10" t="str">
         <x:f>IF(TRIM($A28)="","",IF(COUNTIF($Q28:$AK28,"?*")=0,"OK","Falta revisar: "&amp;$Q28&amp;$R28&amp;$S28&amp;$T28&amp;$U28&amp;$V28&amp;$W28&amp;$X28&amp;$Y28&amp;$Z28&amp;$AA28&amp;$AB28&amp;$AC28&amp;$AD28&amp;$AE28&amp;$AF28&amp;$AG28&amp;$AH28&amp;$AI28&amp;$AJ28&amp;$AK28))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M28"/>
       <x:c r="N28"/>
       <x:c r="O28"/>
       <x:c r="P28"/>
@@ -4763,11 +4771,11 @@
       <x:c r="K29" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L29" s="10"/>
-      <x:c r="M29" t="str">
+      <x:c r="L29" s="10" t="str">
         <x:f>IF(TRIM($A29)="","",IF(COUNTIF($Q29:$AK29,"?*")=0,"OK","Falta revisar: "&amp;$Q29&amp;$R29&amp;$S29&amp;$T29&amp;$U29&amp;$V29&amp;$W29&amp;$X29&amp;$Y29&amp;$Z29&amp;$AA29&amp;$AB29&amp;$AC29&amp;$AD29&amp;$AE29&amp;$AF29&amp;$AG29&amp;$AH29&amp;$AI29&amp;$AJ29&amp;$AK29))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M29"/>
       <x:c r="N29"/>
       <x:c r="O29"/>
       <x:c r="P29"/>
@@ -4879,11 +4887,11 @@
       <x:c r="K30" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L30" s="10"/>
-      <x:c r="M30" t="str">
+      <x:c r="L30" s="10" t="str">
         <x:f>IF(TRIM($A30)="","",IF(COUNTIF($Q30:$AK30,"?*")=0,"OK","Falta revisar: "&amp;$Q30&amp;$R30&amp;$S30&amp;$T30&amp;$U30&amp;$V30&amp;$W30&amp;$X30&amp;$Y30&amp;$Z30&amp;$AA30&amp;$AB30&amp;$AC30&amp;$AD30&amp;$AE30&amp;$AF30&amp;$AG30&amp;$AH30&amp;$AI30&amp;$AJ30&amp;$AK30))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M30"/>
       <x:c r="N30"/>
       <x:c r="O30"/>
       <x:c r="P30"/>
@@ -4995,11 +5003,11 @@
       <x:c r="K31" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L31" s="10"/>
-      <x:c r="M31" t="str">
+      <x:c r="L31" s="10" t="str">
         <x:f>IF(TRIM($A31)="","",IF(COUNTIF($Q31:$AK31,"?*")=0,"OK","Falta revisar: "&amp;$Q31&amp;$R31&amp;$S31&amp;$T31&amp;$U31&amp;$V31&amp;$W31&amp;$X31&amp;$Y31&amp;$Z31&amp;$AA31&amp;$AB31&amp;$AC31&amp;$AD31&amp;$AE31&amp;$AF31&amp;$AG31&amp;$AH31&amp;$AI31&amp;$AJ31&amp;$AK31))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M31"/>
       <x:c r="N31"/>
       <x:c r="O31"/>
       <x:c r="P31"/>
@@ -5111,11 +5119,11 @@
       <x:c r="K32" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L32" s="13"/>
-      <x:c r="M32" t="str">
+      <x:c r="L32" s="13" t="str">
         <x:f>IF(TRIM($A32)="","",IF(COUNTIF($Q32:$AK32,"?*")=0,"OK","Falta revisar: "&amp;$Q32&amp;$R32&amp;$S32&amp;$T32&amp;$U32&amp;$V32&amp;$W32&amp;$X32&amp;$Y32&amp;$Z32&amp;$AA32&amp;$AB32&amp;$AC32&amp;$AD32&amp;$AE32&amp;$AF32&amp;$AG32&amp;$AH32&amp;$AI32&amp;$AJ32&amp;$AK32))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M32"/>
       <x:c r="N32"/>
       <x:c r="O32"/>
       <x:c r="P32"/>
@@ -5227,11 +5235,11 @@
       <x:c r="K33" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L33" s="13"/>
-      <x:c r="M33" t="str">
+      <x:c r="L33" s="13" t="str">
         <x:f>IF(TRIM($A33)="","",IF(COUNTIF($Q33:$AK33,"?*")=0,"OK","Falta revisar: "&amp;$Q33&amp;$R33&amp;$S33&amp;$T33&amp;$U33&amp;$V33&amp;$W33&amp;$X33&amp;$Y33&amp;$Z33&amp;$AA33&amp;$AB33&amp;$AC33&amp;$AD33&amp;$AE33&amp;$AF33&amp;$AG33&amp;$AH33&amp;$AI33&amp;$AJ33&amp;$AK33))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M33"/>
       <x:c r="N33"/>
       <x:c r="O33"/>
       <x:c r="P33"/>
@@ -5343,11 +5351,11 @@
       <x:c r="K34" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L34" s="13"/>
-      <x:c r="M34" t="str">
+      <x:c r="L34" s="13" t="str">
         <x:f>IF(TRIM($A34)="","",IF(COUNTIF($Q34:$AK34,"?*")=0,"OK","Falta revisar: "&amp;$Q34&amp;$R34&amp;$S34&amp;$T34&amp;$U34&amp;$V34&amp;$W34&amp;$X34&amp;$Y34&amp;$Z34&amp;$AA34&amp;$AB34&amp;$AC34&amp;$AD34&amp;$AE34&amp;$AF34&amp;$AG34&amp;$AH34&amp;$AI34&amp;$AJ34&amp;$AK34))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M34"/>
       <x:c r="N34"/>
       <x:c r="O34"/>
       <x:c r="P34"/>
@@ -5459,11 +5467,11 @@
       <x:c r="K35" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L35" s="13"/>
-      <x:c r="M35" t="str">
+      <x:c r="L35" s="13" t="str">
         <x:f>IF(TRIM($A35)="","",IF(COUNTIF($Q35:$AK35,"?*")=0,"OK","Falta revisar: "&amp;$Q35&amp;$R35&amp;$S35&amp;$T35&amp;$U35&amp;$V35&amp;$W35&amp;$X35&amp;$Y35&amp;$Z35&amp;$AA35&amp;$AB35&amp;$AC35&amp;$AD35&amp;$AE35&amp;$AF35&amp;$AG35&amp;$AH35&amp;$AI35&amp;$AJ35&amp;$AK35))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M35"/>
       <x:c r="N35"/>
       <x:c r="O35"/>
       <x:c r="P35"/>
@@ -5575,11 +5583,11 @@
       <x:c r="K36" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L36" s="13"/>
-      <x:c r="M36" t="str">
+      <x:c r="L36" s="13" t="str">
         <x:f>IF(TRIM($A36)="","",IF(COUNTIF($Q36:$AK36,"?*")=0,"OK","Falta revisar: "&amp;$Q36&amp;$R36&amp;$S36&amp;$T36&amp;$U36&amp;$V36&amp;$W36&amp;$X36&amp;$Y36&amp;$Z36&amp;$AA36&amp;$AB36&amp;$AC36&amp;$AD36&amp;$AE36&amp;$AF36&amp;$AG36&amp;$AH36&amp;$AI36&amp;$AJ36&amp;$AK36))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M36"/>
       <x:c r="N36"/>
       <x:c r="O36"/>
       <x:c r="P36"/>
@@ -5691,11 +5699,11 @@
       <x:c r="K37" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L37" s="13"/>
-      <x:c r="M37" t="str">
+      <x:c r="L37" s="13" t="str">
         <x:f>IF(TRIM($A37)="","",IF(COUNTIF($Q37:$AK37,"?*")=0,"OK","Falta revisar: "&amp;$Q37&amp;$R37&amp;$S37&amp;$T37&amp;$U37&amp;$V37&amp;$W37&amp;$X37&amp;$Y37&amp;$Z37&amp;$AA37&amp;$AB37&amp;$AC37&amp;$AD37&amp;$AE37&amp;$AF37&amp;$AG37&amp;$AH37&amp;$AI37&amp;$AJ37&amp;$AK37))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M37"/>
       <x:c r="N37"/>
       <x:c r="O37"/>
       <x:c r="P37"/>
@@ -5807,11 +5815,11 @@
       <x:c r="K38" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L38" s="13"/>
-      <x:c r="M38" t="str">
+      <x:c r="L38" s="13" t="str">
         <x:f>IF(TRIM($A38)="","",IF(COUNTIF($Q38:$AK38,"?*")=0,"OK","Falta revisar: "&amp;$Q38&amp;$R38&amp;$S38&amp;$T38&amp;$U38&amp;$V38&amp;$W38&amp;$X38&amp;$Y38&amp;$Z38&amp;$AA38&amp;$AB38&amp;$AC38&amp;$AD38&amp;$AE38&amp;$AF38&amp;$AG38&amp;$AH38&amp;$AI38&amp;$AJ38&amp;$AK38))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M38"/>
       <x:c r="N38"/>
       <x:c r="O38"/>
       <x:c r="P38"/>
@@ -5923,11 +5931,11 @@
       <x:c r="K39" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L39" s="13"/>
-      <x:c r="M39" t="str">
+      <x:c r="L39" s="13" t="str">
         <x:f>IF(TRIM($A39)="","",IF(COUNTIF($Q39:$AK39,"?*")=0,"OK","Falta revisar: "&amp;$Q39&amp;$R39&amp;$S39&amp;$T39&amp;$U39&amp;$V39&amp;$W39&amp;$X39&amp;$Y39&amp;$Z39&amp;$AA39&amp;$AB39&amp;$AC39&amp;$AD39&amp;$AE39&amp;$AF39&amp;$AG39&amp;$AH39&amp;$AI39&amp;$AJ39&amp;$AK39))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M39"/>
       <x:c r="N39"/>
       <x:c r="O39"/>
       <x:c r="P39"/>
@@ -6039,11 +6047,11 @@
       <x:c r="K40" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L40" s="13"/>
-      <x:c r="M40" t="str">
+      <x:c r="L40" s="13" t="str">
         <x:f>IF(TRIM($A40)="","",IF(COUNTIF($Q40:$AK40,"?*")=0,"OK","Falta revisar: "&amp;$Q40&amp;$R40&amp;$S40&amp;$T40&amp;$U40&amp;$V40&amp;$W40&amp;$X40&amp;$Y40&amp;$Z40&amp;$AA40&amp;$AB40&amp;$AC40&amp;$AD40&amp;$AE40&amp;$AF40&amp;$AG40&amp;$AH40&amp;$AI40&amp;$AJ40&amp;$AK40))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M40"/>
       <x:c r="N40"/>
       <x:c r="O40"/>
       <x:c r="P40"/>
@@ -6155,11 +6163,11 @@
       <x:c r="K41" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L41" s="13"/>
-      <x:c r="M41" t="str">
+      <x:c r="L41" s="13" t="str">
         <x:f>IF(TRIM($A41)="","",IF(COUNTIF($Q41:$AK41,"?*")=0,"OK","Falta revisar: "&amp;$Q41&amp;$R41&amp;$S41&amp;$T41&amp;$U41&amp;$V41&amp;$W41&amp;$X41&amp;$Y41&amp;$Z41&amp;$AA41&amp;$AB41&amp;$AC41&amp;$AD41&amp;$AE41&amp;$AF41&amp;$AG41&amp;$AH41&amp;$AI41&amp;$AJ41&amp;$AK41))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M41"/>
       <x:c r="N41"/>
       <x:c r="O41"/>
       <x:c r="P41"/>
@@ -6271,11 +6279,11 @@
       <x:c r="K42" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L42" s="13"/>
-      <x:c r="M42" t="str">
+      <x:c r="L42" s="13" t="str">
         <x:f>IF(TRIM($A42)="","",IF(COUNTIF($Q42:$AK42,"?*")=0,"OK","Falta revisar: "&amp;$Q42&amp;$R42&amp;$S42&amp;$T42&amp;$U42&amp;$V42&amp;$W42&amp;$X42&amp;$Y42&amp;$Z42&amp;$AA42&amp;$AB42&amp;$AC42&amp;$AD42&amp;$AE42&amp;$AF42&amp;$AG42&amp;$AH42&amp;$AI42&amp;$AJ42&amp;$AK42))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M42"/>
       <x:c r="N42"/>
       <x:c r="O42"/>
       <x:c r="P42"/>
@@ -6387,11 +6395,11 @@
       <x:c r="K43" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L43" s="13"/>
-      <x:c r="M43" t="str">
+      <x:c r="L43" s="13" t="str">
         <x:f>IF(TRIM($A43)="","",IF(COUNTIF($Q43:$AK43,"?*")=0,"OK","Falta revisar: "&amp;$Q43&amp;$R43&amp;$S43&amp;$T43&amp;$U43&amp;$V43&amp;$W43&amp;$X43&amp;$Y43&amp;$Z43&amp;$AA43&amp;$AB43&amp;$AC43&amp;$AD43&amp;$AE43&amp;$AF43&amp;$AG43&amp;$AH43&amp;$AI43&amp;$AJ43&amp;$AK43))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M43"/>
       <x:c r="N43"/>
       <x:c r="O43"/>
       <x:c r="P43"/>
@@ -6503,11 +6511,11 @@
       <x:c r="K44" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L44" s="13"/>
-      <x:c r="M44" t="str">
+      <x:c r="L44" s="13" t="str">
         <x:f>IF(TRIM($A44)="","",IF(COUNTIF($Q44:$AK44,"?*")=0,"OK","Falta revisar: "&amp;$Q44&amp;$R44&amp;$S44&amp;$T44&amp;$U44&amp;$V44&amp;$W44&amp;$X44&amp;$Y44&amp;$Z44&amp;$AA44&amp;$AB44&amp;$AC44&amp;$AD44&amp;$AE44&amp;$AF44&amp;$AG44&amp;$AH44&amp;$AI44&amp;$AJ44&amp;$AK44))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M44"/>
       <x:c r="N44"/>
       <x:c r="O44"/>
       <x:c r="P44"/>
@@ -6619,11 +6627,11 @@
       <x:c r="K45" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L45" s="13"/>
-      <x:c r="M45" t="str">
+      <x:c r="L45" s="13" t="str">
         <x:f>IF(TRIM($A45)="","",IF(COUNTIF($Q45:$AK45,"?*")=0,"OK","Falta revisar: "&amp;$Q45&amp;$R45&amp;$S45&amp;$T45&amp;$U45&amp;$V45&amp;$W45&amp;$X45&amp;$Y45&amp;$Z45&amp;$AA45&amp;$AB45&amp;$AC45&amp;$AD45&amp;$AE45&amp;$AF45&amp;$AG45&amp;$AH45&amp;$AI45&amp;$AJ45&amp;$AK45))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M45"/>
       <x:c r="N45"/>
       <x:c r="O45"/>
       <x:c r="P45"/>
@@ -6735,11 +6743,11 @@
       <x:c r="K46" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L46" s="13"/>
-      <x:c r="M46" t="str">
+      <x:c r="L46" s="13" t="str">
         <x:f>IF(TRIM($A46)="","",IF(COUNTIF($Q46:$AK46,"?*")=0,"OK","Falta revisar: "&amp;$Q46&amp;$R46&amp;$S46&amp;$T46&amp;$U46&amp;$V46&amp;$W46&amp;$X46&amp;$Y46&amp;$Z46&amp;$AA46&amp;$AB46&amp;$AC46&amp;$AD46&amp;$AE46&amp;$AF46&amp;$AG46&amp;$AH46&amp;$AI46&amp;$AJ46&amp;$AK46))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M46"/>
       <x:c r="N46"/>
       <x:c r="O46"/>
       <x:c r="P46"/>
@@ -6851,11 +6859,11 @@
       <x:c r="K47" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L47" s="13"/>
-      <x:c r="M47" t="str">
+      <x:c r="L47" s="13" t="str">
         <x:f>IF(TRIM($A47)="","",IF(COUNTIF($Q47:$AK47,"?*")=0,"OK","Falta revisar: "&amp;$Q47&amp;$R47&amp;$S47&amp;$T47&amp;$U47&amp;$V47&amp;$W47&amp;$X47&amp;$Y47&amp;$Z47&amp;$AA47&amp;$AB47&amp;$AC47&amp;$AD47&amp;$AE47&amp;$AF47&amp;$AG47&amp;$AH47&amp;$AI47&amp;$AJ47&amp;$AK47))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M47"/>
       <x:c r="N47"/>
       <x:c r="O47"/>
       <x:c r="P47"/>
@@ -6967,11 +6975,11 @@
       <x:c r="K48" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L48" s="13"/>
-      <x:c r="M48" t="str">
+      <x:c r="L48" s="13" t="str">
         <x:f>IF(TRIM($A48)="","",IF(COUNTIF($Q48:$AK48,"?*")=0,"OK","Falta revisar: "&amp;$Q48&amp;$R48&amp;$S48&amp;$T48&amp;$U48&amp;$V48&amp;$W48&amp;$X48&amp;$Y48&amp;$Z48&amp;$AA48&amp;$AB48&amp;$AC48&amp;$AD48&amp;$AE48&amp;$AF48&amp;$AG48&amp;$AH48&amp;$AI48&amp;$AJ48&amp;$AK48))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M48"/>
       <x:c r="N48"/>
       <x:c r="O48"/>
       <x:c r="P48"/>
@@ -7083,11 +7091,11 @@
       <x:c r="K49" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L49" s="13"/>
-      <x:c r="M49" t="str">
+      <x:c r="L49" s="13" t="str">
         <x:f>IF(TRIM($A49)="","",IF(COUNTIF($Q49:$AK49,"?*")=0,"OK","Falta revisar: "&amp;$Q49&amp;$R49&amp;$S49&amp;$T49&amp;$U49&amp;$V49&amp;$W49&amp;$X49&amp;$Y49&amp;$Z49&amp;$AA49&amp;$AB49&amp;$AC49&amp;$AD49&amp;$AE49&amp;$AF49&amp;$AG49&amp;$AH49&amp;$AI49&amp;$AJ49&amp;$AK49))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M49"/>
       <x:c r="N49"/>
       <x:c r="O49"/>
       <x:c r="P49"/>
@@ -7199,11 +7207,11 @@
       <x:c r="K50" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L50" s="13"/>
-      <x:c r="M50" t="str">
+      <x:c r="L50" s="13" t="str">
         <x:f>IF(TRIM($A50)="","",IF(COUNTIF($Q50:$AK50,"?*")=0,"OK","Falta revisar: "&amp;$Q50&amp;$R50&amp;$S50&amp;$T50&amp;$U50&amp;$V50&amp;$W50&amp;$X50&amp;$Y50&amp;$Z50&amp;$AA50&amp;$AB50&amp;$AC50&amp;$AD50&amp;$AE50&amp;$AF50&amp;$AG50&amp;$AH50&amp;$AI50&amp;$AJ50&amp;$AK50))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M50"/>
       <x:c r="N50"/>
       <x:c r="O50"/>
       <x:c r="P50"/>
@@ -7315,11 +7323,11 @@
       <x:c r="K51" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L51" s="13"/>
-      <x:c r="M51" t="str">
+      <x:c r="L51" s="13" t="str">
         <x:f>IF(TRIM($A51)="","",IF(COUNTIF($Q51:$AK51,"?*")=0,"OK","Falta revisar: "&amp;$Q51&amp;$R51&amp;$S51&amp;$T51&amp;$U51&amp;$V51&amp;$W51&amp;$X51&amp;$Y51&amp;$Z51&amp;$AA51&amp;$AB51&amp;$AC51&amp;$AD51&amp;$AE51&amp;$AF51&amp;$AG51&amp;$AH51&amp;$AI51&amp;$AJ51&amp;$AK51))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M51"/>
       <x:c r="N51"/>
       <x:c r="O51"/>
       <x:c r="P51"/>
@@ -7431,11 +7439,11 @@
       <x:c r="K52" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L52" s="13"/>
-      <x:c r="M52" t="str">
+      <x:c r="L52" s="13" t="str">
         <x:f>IF(TRIM($A52)="","",IF(COUNTIF($Q52:$AK52,"?*")=0,"OK","Falta revisar: "&amp;$Q52&amp;$R52&amp;$S52&amp;$T52&amp;$U52&amp;$V52&amp;$W52&amp;$X52&amp;$Y52&amp;$Z52&amp;$AA52&amp;$AB52&amp;$AC52&amp;$AD52&amp;$AE52&amp;$AF52&amp;$AG52&amp;$AH52&amp;$AI52&amp;$AJ52&amp;$AK52))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M52"/>
       <x:c r="N52"/>
       <x:c r="O52"/>
       <x:c r="P52"/>
@@ -7547,11 +7555,11 @@
       <x:c r="K53" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L53" s="13"/>
-      <x:c r="M53" t="str">
+      <x:c r="L53" s="13" t="str">
         <x:f>IF(TRIM($A53)="","",IF(COUNTIF($Q53:$AK53,"?*")=0,"OK","Falta revisar: "&amp;$Q53&amp;$R53&amp;$S53&amp;$T53&amp;$U53&amp;$V53&amp;$W53&amp;$X53&amp;$Y53&amp;$Z53&amp;$AA53&amp;$AB53&amp;$AC53&amp;$AD53&amp;$AE53&amp;$AF53&amp;$AG53&amp;$AH53&amp;$AI53&amp;$AJ53&amp;$AK53))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M53"/>
       <x:c r="N53"/>
       <x:c r="O53"/>
       <x:c r="P53"/>
@@ -7663,11 +7671,11 @@
       <x:c r="K54" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L54" s="13"/>
-      <x:c r="M54" t="str">
+      <x:c r="L54" s="13" t="str">
         <x:f>IF(TRIM($A54)="","",IF(COUNTIF($Q54:$AK54,"?*")=0,"OK","Falta revisar: "&amp;$Q54&amp;$R54&amp;$S54&amp;$T54&amp;$U54&amp;$V54&amp;$W54&amp;$X54&amp;$Y54&amp;$Z54&amp;$AA54&amp;$AB54&amp;$AC54&amp;$AD54&amp;$AE54&amp;$AF54&amp;$AG54&amp;$AH54&amp;$AI54&amp;$AJ54&amp;$AK54))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M54"/>
       <x:c r="N54"/>
       <x:c r="O54"/>
       <x:c r="P54"/>
@@ -7779,11 +7787,11 @@
       <x:c r="K55" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L55" s="13"/>
-      <x:c r="M55" t="str">
+      <x:c r="L55" s="13" t="str">
         <x:f>IF(TRIM($A55)="","",IF(COUNTIF($Q55:$AK55,"?*")=0,"OK","Falta revisar: "&amp;$Q55&amp;$R55&amp;$S55&amp;$T55&amp;$U55&amp;$V55&amp;$W55&amp;$X55&amp;$Y55&amp;$Z55&amp;$AA55&amp;$AB55&amp;$AC55&amp;$AD55&amp;$AE55&amp;$AF55&amp;$AG55&amp;$AH55&amp;$AI55&amp;$AJ55&amp;$AK55))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M55"/>
       <x:c r="N55"/>
       <x:c r="O55"/>
       <x:c r="P55"/>
@@ -7895,11 +7903,11 @@
       <x:c r="K56" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L56" s="13"/>
-      <x:c r="M56" t="str">
+      <x:c r="L56" s="13" t="str">
         <x:f>IF(TRIM($A56)="","",IF(COUNTIF($Q56:$AK56,"?*")=0,"OK","Falta revisar: "&amp;$Q56&amp;$R56&amp;$S56&amp;$T56&amp;$U56&amp;$V56&amp;$W56&amp;$X56&amp;$Y56&amp;$Z56&amp;$AA56&amp;$AB56&amp;$AC56&amp;$AD56&amp;$AE56&amp;$AF56&amp;$AG56&amp;$AH56&amp;$AI56&amp;$AJ56&amp;$AK56))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M56"/>
       <x:c r="N56"/>
       <x:c r="O56"/>
       <x:c r="P56"/>
@@ -8011,11 +8019,11 @@
       <x:c r="K57" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L57" s="13"/>
-      <x:c r="M57" t="str">
+      <x:c r="L57" s="13" t="str">
         <x:f>IF(TRIM($A57)="","",IF(COUNTIF($Q57:$AK57,"?*")=0,"OK","Falta revisar: "&amp;$Q57&amp;$R57&amp;$S57&amp;$T57&amp;$U57&amp;$V57&amp;$W57&amp;$X57&amp;$Y57&amp;$Z57&amp;$AA57&amp;$AB57&amp;$AC57&amp;$AD57&amp;$AE57&amp;$AF57&amp;$AG57&amp;$AH57&amp;$AI57&amp;$AJ57&amp;$AK57))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M57"/>
       <x:c r="N57"/>
       <x:c r="O57"/>
       <x:c r="P57"/>
@@ -8127,11 +8135,11 @@
       <x:c r="K58" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L58" s="13"/>
-      <x:c r="M58" t="str">
+      <x:c r="L58" s="13" t="str">
         <x:f>IF(TRIM($A58)="","",IF(COUNTIF($Q58:$AK58,"?*")=0,"OK","Falta revisar: "&amp;$Q58&amp;$R58&amp;$S58&amp;$T58&amp;$U58&amp;$V58&amp;$W58&amp;$X58&amp;$Y58&amp;$Z58&amp;$AA58&amp;$AB58&amp;$AC58&amp;$AD58&amp;$AE58&amp;$AF58&amp;$AG58&amp;$AH58&amp;$AI58&amp;$AJ58&amp;$AK58))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M58"/>
       <x:c r="N58"/>
       <x:c r="O58"/>
       <x:c r="P58"/>
@@ -8243,11 +8251,11 @@
       <x:c r="K59" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L59" s="13"/>
-      <x:c r="M59" t="str">
+      <x:c r="L59" s="13" t="str">
         <x:f>IF(TRIM($A59)="","",IF(COUNTIF($Q59:$AK59,"?*")=0,"OK","Falta revisar: "&amp;$Q59&amp;$R59&amp;$S59&amp;$T59&amp;$U59&amp;$V59&amp;$W59&amp;$X59&amp;$Y59&amp;$Z59&amp;$AA59&amp;$AB59&amp;$AC59&amp;$AD59&amp;$AE59&amp;$AF59&amp;$AG59&amp;$AH59&amp;$AI59&amp;$AJ59&amp;$AK59))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M59"/>
       <x:c r="N59"/>
       <x:c r="O59"/>
       <x:c r="P59"/>
@@ -8359,11 +8367,11 @@
       <x:c r="K60" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L60" s="13"/>
-      <x:c r="M60" t="str">
+      <x:c r="L60" s="13" t="str">
         <x:f>IF(TRIM($A60)="","",IF(COUNTIF($Q60:$AK60,"?*")=0,"OK","Falta revisar: "&amp;$Q60&amp;$R60&amp;$S60&amp;$T60&amp;$U60&amp;$V60&amp;$W60&amp;$X60&amp;$Y60&amp;$Z60&amp;$AA60&amp;$AB60&amp;$AC60&amp;$AD60&amp;$AE60&amp;$AF60&amp;$AG60&amp;$AH60&amp;$AI60&amp;$AJ60&amp;$AK60))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M60"/>
       <x:c r="N60"/>
       <x:c r="O60"/>
       <x:c r="P60"/>
@@ -8475,11 +8483,11 @@
       <x:c r="K61" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L61" s="13"/>
-      <x:c r="M61" t="str">
+      <x:c r="L61" s="13" t="str">
         <x:f>IF(TRIM($A61)="","",IF(COUNTIF($Q61:$AK61,"?*")=0,"OK","Falta revisar: "&amp;$Q61&amp;$R61&amp;$S61&amp;$T61&amp;$U61&amp;$V61&amp;$W61&amp;$X61&amp;$Y61&amp;$Z61&amp;$AA61&amp;$AB61&amp;$AC61&amp;$AD61&amp;$AE61&amp;$AF61&amp;$AG61&amp;$AH61&amp;$AI61&amp;$AJ61&amp;$AK61))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M61"/>
       <x:c r="N61"/>
       <x:c r="O61"/>
       <x:c r="P61"/>
@@ -8591,11 +8599,11 @@
       <x:c r="K62" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L62" s="13"/>
-      <x:c r="M62" t="str">
+      <x:c r="L62" s="13" t="str">
         <x:f>IF(TRIM($A62)="","",IF(COUNTIF($Q62:$AK62,"?*")=0,"OK","Falta revisar: "&amp;$Q62&amp;$R62&amp;$S62&amp;$T62&amp;$U62&amp;$V62&amp;$W62&amp;$X62&amp;$Y62&amp;$Z62&amp;$AA62&amp;$AB62&amp;$AC62&amp;$AD62&amp;$AE62&amp;$AF62&amp;$AG62&amp;$AH62&amp;$AI62&amp;$AJ62&amp;$AK62))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M62"/>
       <x:c r="N62"/>
       <x:c r="O62"/>
       <x:c r="P62"/>
@@ -8707,11 +8715,11 @@
       <x:c r="K63" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L63" s="13"/>
-      <x:c r="M63" t="str">
+      <x:c r="L63" s="13" t="str">
         <x:f>IF(TRIM($A63)="","",IF(COUNTIF($Q63:$AK63,"?*")=0,"OK","Falta revisar: "&amp;$Q63&amp;$R63&amp;$S63&amp;$T63&amp;$U63&amp;$V63&amp;$W63&amp;$X63&amp;$Y63&amp;$Z63&amp;$AA63&amp;$AB63&amp;$AC63&amp;$AD63&amp;$AE63&amp;$AF63&amp;$AG63&amp;$AH63&amp;$AI63&amp;$AJ63&amp;$AK63))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M63"/>
       <x:c r="N63"/>
       <x:c r="O63"/>
       <x:c r="P63"/>
@@ -8823,11 +8831,11 @@
       <x:c r="K64" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L64" s="13"/>
-      <x:c r="M64" t="str">
+      <x:c r="L64" s="13" t="str">
         <x:f>IF(TRIM($A64)="","",IF(COUNTIF($Q64:$AK64,"?*")=0,"OK","Falta revisar: "&amp;$Q64&amp;$R64&amp;$S64&amp;$T64&amp;$U64&amp;$V64&amp;$W64&amp;$X64&amp;$Y64&amp;$Z64&amp;$AA64&amp;$AB64&amp;$AC64&amp;$AD64&amp;$AE64&amp;$AF64&amp;$AG64&amp;$AH64&amp;$AI64&amp;$AJ64&amp;$AK64))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M64"/>
       <x:c r="N64"/>
       <x:c r="O64"/>
       <x:c r="P64"/>
@@ -8939,11 +8947,11 @@
       <x:c r="K65" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L65" s="13"/>
-      <x:c r="M65" t="str">
+      <x:c r="L65" s="13" t="str">
         <x:f>IF(TRIM($A65)="","",IF(COUNTIF($Q65:$AK65,"?*")=0,"OK","Falta revisar: "&amp;$Q65&amp;$R65&amp;$S65&amp;$T65&amp;$U65&amp;$V65&amp;$W65&amp;$X65&amp;$Y65&amp;$Z65&amp;$AA65&amp;$AB65&amp;$AC65&amp;$AD65&amp;$AE65&amp;$AF65&amp;$AG65&amp;$AH65&amp;$AI65&amp;$AJ65&amp;$AK65))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M65"/>
       <x:c r="N65"/>
       <x:c r="O65"/>
       <x:c r="P65"/>
@@ -9055,11 +9063,11 @@
       <x:c r="K66" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L66" s="13"/>
-      <x:c r="M66" t="str">
+      <x:c r="L66" s="13" t="str">
         <x:f>IF(TRIM($A66)="","",IF(COUNTIF($Q66:$AK66,"?*")=0,"OK","Falta revisar: "&amp;$Q66&amp;$R66&amp;$S66&amp;$T66&amp;$U66&amp;$V66&amp;$W66&amp;$X66&amp;$Y66&amp;$Z66&amp;$AA66&amp;$AB66&amp;$AC66&amp;$AD66&amp;$AE66&amp;$AF66&amp;$AG66&amp;$AH66&amp;$AI66&amp;$AJ66&amp;$AK66))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M66"/>
       <x:c r="N66"/>
       <x:c r="O66"/>
       <x:c r="P66"/>
@@ -9171,11 +9179,11 @@
       <x:c r="K67" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L67" s="13"/>
-      <x:c r="M67" t="str">
+      <x:c r="L67" s="13" t="str">
         <x:f>IF(TRIM($A67)="","",IF(COUNTIF($Q67:$AK67,"?*")=0,"OK","Falta revisar: "&amp;$Q67&amp;$R67&amp;$S67&amp;$T67&amp;$U67&amp;$V67&amp;$W67&amp;$X67&amp;$Y67&amp;$Z67&amp;$AA67&amp;$AB67&amp;$AC67&amp;$AD67&amp;$AE67&amp;$AF67&amp;$AG67&amp;$AH67&amp;$AI67&amp;$AJ67&amp;$AK67))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M67"/>
       <x:c r="N67"/>
       <x:c r="O67"/>
       <x:c r="P67"/>
@@ -9287,11 +9295,11 @@
       <x:c r="K68" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L68" s="13"/>
-      <x:c r="M68" t="str">
+      <x:c r="L68" s="13" t="str">
         <x:f>IF(TRIM($A68)="","",IF(COUNTIF($Q68:$AK68,"?*")=0,"OK","Falta revisar: "&amp;$Q68&amp;$R68&amp;$S68&amp;$T68&amp;$U68&amp;$V68&amp;$W68&amp;$X68&amp;$Y68&amp;$Z68&amp;$AA68&amp;$AB68&amp;$AC68&amp;$AD68&amp;$AE68&amp;$AF68&amp;$AG68&amp;$AH68&amp;$AI68&amp;$AJ68&amp;$AK68))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M68"/>
       <x:c r="N68"/>
       <x:c r="O68"/>
       <x:c r="P68"/>
@@ -9403,11 +9411,11 @@
       <x:c r="K69" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L69" s="13"/>
-      <x:c r="M69" t="str">
+      <x:c r="L69" s="13" t="str">
         <x:f>IF(TRIM($A69)="","",IF(COUNTIF($Q69:$AK69,"?*")=0,"OK","Falta revisar: "&amp;$Q69&amp;$R69&amp;$S69&amp;$T69&amp;$U69&amp;$V69&amp;$W69&amp;$X69&amp;$Y69&amp;$Z69&amp;$AA69&amp;$AB69&amp;$AC69&amp;$AD69&amp;$AE69&amp;$AF69&amp;$AG69&amp;$AH69&amp;$AI69&amp;$AJ69&amp;$AK69))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M69"/>
       <x:c r="N69"/>
       <x:c r="O69"/>
       <x:c r="P69"/>
@@ -9519,11 +9527,11 @@
       <x:c r="K70" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L70" s="13"/>
-      <x:c r="M70" t="str">
+      <x:c r="L70" s="13" t="str">
         <x:f>IF(TRIM($A70)="","",IF(COUNTIF($Q70:$AK70,"?*")=0,"OK","Falta revisar: "&amp;$Q70&amp;$R70&amp;$S70&amp;$T70&amp;$U70&amp;$V70&amp;$W70&amp;$X70&amp;$Y70&amp;$Z70&amp;$AA70&amp;$AB70&amp;$AC70&amp;$AD70&amp;$AE70&amp;$AF70&amp;$AG70&amp;$AH70&amp;$AI70&amp;$AJ70&amp;$AK70))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M70"/>
       <x:c r="N70"/>
       <x:c r="O70"/>
       <x:c r="P70"/>
@@ -9635,11 +9643,11 @@
       <x:c r="K71" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L71" s="13"/>
-      <x:c r="M71" t="str">
+      <x:c r="L71" s="13" t="str">
         <x:f>IF(TRIM($A71)="","",IF(COUNTIF($Q71:$AK71,"?*")=0,"OK","Falta revisar: "&amp;$Q71&amp;$R71&amp;$S71&amp;$T71&amp;$U71&amp;$V71&amp;$W71&amp;$X71&amp;$Y71&amp;$Z71&amp;$AA71&amp;$AB71&amp;$AC71&amp;$AD71&amp;$AE71&amp;$AF71&amp;$AG71&amp;$AH71&amp;$AI71&amp;$AJ71&amp;$AK71))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M71"/>
       <x:c r="N71"/>
       <x:c r="O71"/>
       <x:c r="P71"/>
@@ -9751,11 +9759,11 @@
       <x:c r="K72" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L72" s="13"/>
-      <x:c r="M72" t="str">
+      <x:c r="L72" s="13" t="str">
         <x:f>IF(TRIM($A72)="","",IF(COUNTIF($Q72:$AK72,"?*")=0,"OK","Falta revisar: "&amp;$Q72&amp;$R72&amp;$S72&amp;$T72&amp;$U72&amp;$V72&amp;$W72&amp;$X72&amp;$Y72&amp;$Z72&amp;$AA72&amp;$AB72&amp;$AC72&amp;$AD72&amp;$AE72&amp;$AF72&amp;$AG72&amp;$AH72&amp;$AI72&amp;$AJ72&amp;$AK72))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M72"/>
       <x:c r="N72"/>
       <x:c r="O72"/>
       <x:c r="P72"/>
@@ -9867,11 +9875,11 @@
       <x:c r="K73" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L73" s="13"/>
-      <x:c r="M73" t="str">
+      <x:c r="L73" s="13" t="str">
         <x:f>IF(TRIM($A73)="","",IF(COUNTIF($Q73:$AK73,"?*")=0,"OK","Falta revisar: "&amp;$Q73&amp;$R73&amp;$S73&amp;$T73&amp;$U73&amp;$V73&amp;$W73&amp;$X73&amp;$Y73&amp;$Z73&amp;$AA73&amp;$AB73&amp;$AC73&amp;$AD73&amp;$AE73&amp;$AF73&amp;$AG73&amp;$AH73&amp;$AI73&amp;$AJ73&amp;$AK73))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M73"/>
       <x:c r="N73"/>
       <x:c r="O73"/>
       <x:c r="P73"/>
@@ -9983,11 +9991,11 @@
       <x:c r="K74" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L74" s="13"/>
-      <x:c r="M74" t="str">
+      <x:c r="L74" s="13" t="str">
         <x:f>IF(TRIM($A74)="","",IF(COUNTIF($Q74:$AK74,"?*")=0,"OK","Falta revisar: "&amp;$Q74&amp;$R74&amp;$S74&amp;$T74&amp;$U74&amp;$V74&amp;$W74&amp;$X74&amp;$Y74&amp;$Z74&amp;$AA74&amp;$AB74&amp;$AC74&amp;$AD74&amp;$AE74&amp;$AF74&amp;$AG74&amp;$AH74&amp;$AI74&amp;$AJ74&amp;$AK74))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M74"/>
       <x:c r="N74"/>
       <x:c r="O74"/>
       <x:c r="P74"/>
@@ -10099,11 +10107,11 @@
       <x:c r="K75" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L75" s="13"/>
-      <x:c r="M75" t="str">
+      <x:c r="L75" s="13" t="str">
         <x:f>IF(TRIM($A75)="","",IF(COUNTIF($Q75:$AK75,"?*")=0,"OK","Falta revisar: "&amp;$Q75&amp;$R75&amp;$S75&amp;$T75&amp;$U75&amp;$V75&amp;$W75&amp;$X75&amp;$Y75&amp;$Z75&amp;$AA75&amp;$AB75&amp;$AC75&amp;$AD75&amp;$AE75&amp;$AF75&amp;$AG75&amp;$AH75&amp;$AI75&amp;$AJ75&amp;$AK75))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M75"/>
       <x:c r="N75"/>
       <x:c r="O75"/>
       <x:c r="P75"/>
@@ -10215,11 +10223,11 @@
       <x:c r="K76" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L76" s="13"/>
-      <x:c r="M76" t="str">
+      <x:c r="L76" s="13" t="str">
         <x:f>IF(TRIM($A76)="","",IF(COUNTIF($Q76:$AK76,"?*")=0,"OK","Falta revisar: "&amp;$Q76&amp;$R76&amp;$S76&amp;$T76&amp;$U76&amp;$V76&amp;$W76&amp;$X76&amp;$Y76&amp;$Z76&amp;$AA76&amp;$AB76&amp;$AC76&amp;$AD76&amp;$AE76&amp;$AF76&amp;$AG76&amp;$AH76&amp;$AI76&amp;$AJ76&amp;$AK76))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M76"/>
       <x:c r="N76"/>
       <x:c r="O76"/>
       <x:c r="P76"/>
@@ -10331,11 +10339,11 @@
       <x:c r="K77" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L77" s="13"/>
-      <x:c r="M77" t="str">
+      <x:c r="L77" s="13" t="str">
         <x:f>IF(TRIM($A77)="","",IF(COUNTIF($Q77:$AK77,"?*")=0,"OK","Falta revisar: "&amp;$Q77&amp;$R77&amp;$S77&amp;$T77&amp;$U77&amp;$V77&amp;$W77&amp;$X77&amp;$Y77&amp;$Z77&amp;$AA77&amp;$AB77&amp;$AC77&amp;$AD77&amp;$AE77&amp;$AF77&amp;$AG77&amp;$AH77&amp;$AI77&amp;$AJ77&amp;$AK77))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M77"/>
       <x:c r="N77"/>
       <x:c r="O77"/>
       <x:c r="P77"/>
@@ -10447,11 +10455,11 @@
       <x:c r="K78" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L78" s="13"/>
-      <x:c r="M78" t="str">
+      <x:c r="L78" s="13" t="str">
         <x:f>IF(TRIM($A78)="","",IF(COUNTIF($Q78:$AK78,"?*")=0,"OK","Falta revisar: "&amp;$Q78&amp;$R78&amp;$S78&amp;$T78&amp;$U78&amp;$V78&amp;$W78&amp;$X78&amp;$Y78&amp;$Z78&amp;$AA78&amp;$AB78&amp;$AC78&amp;$AD78&amp;$AE78&amp;$AF78&amp;$AG78&amp;$AH78&amp;$AI78&amp;$AJ78&amp;$AK78))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M78"/>
       <x:c r="N78"/>
       <x:c r="O78"/>
       <x:c r="P78"/>
@@ -10563,11 +10571,11 @@
       <x:c r="K79" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L79" s="13"/>
-      <x:c r="M79" t="str">
+      <x:c r="L79" s="13" t="str">
         <x:f>IF(TRIM($A79)="","",IF(COUNTIF($Q79:$AK79,"?*")=0,"OK","Falta revisar: "&amp;$Q79&amp;$R79&amp;$S79&amp;$T79&amp;$U79&amp;$V79&amp;$W79&amp;$X79&amp;$Y79&amp;$Z79&amp;$AA79&amp;$AB79&amp;$AC79&amp;$AD79&amp;$AE79&amp;$AF79&amp;$AG79&amp;$AH79&amp;$AI79&amp;$AJ79&amp;$AK79))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M79"/>
       <x:c r="N79"/>
       <x:c r="O79"/>
       <x:c r="P79"/>
@@ -10679,11 +10687,11 @@
       <x:c r="K80" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L80" s="13"/>
-      <x:c r="M80" t="str">
+      <x:c r="L80" s="13" t="str">
         <x:f>IF(TRIM($A80)="","",IF(COUNTIF($Q80:$AK80,"?*")=0,"OK","Falta revisar: "&amp;$Q80&amp;$R80&amp;$S80&amp;$T80&amp;$U80&amp;$V80&amp;$W80&amp;$X80&amp;$Y80&amp;$Z80&amp;$AA80&amp;$AB80&amp;$AC80&amp;$AD80&amp;$AE80&amp;$AF80&amp;$AG80&amp;$AH80&amp;$AI80&amp;$AJ80&amp;$AK80))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M80"/>
       <x:c r="N80"/>
       <x:c r="O80"/>
       <x:c r="P80"/>
@@ -10795,11 +10803,11 @@
       <x:c r="K81" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L81" s="13"/>
-      <x:c r="M81" t="str">
+      <x:c r="L81" s="13" t="str">
         <x:f>IF(TRIM($A81)="","",IF(COUNTIF($Q81:$AK81,"?*")=0,"OK","Falta revisar: "&amp;$Q81&amp;$R81&amp;$S81&amp;$T81&amp;$U81&amp;$V81&amp;$W81&amp;$X81&amp;$Y81&amp;$Z81&amp;$AA81&amp;$AB81&amp;$AC81&amp;$AD81&amp;$AE81&amp;$AF81&amp;$AG81&amp;$AH81&amp;$AI81&amp;$AJ81&amp;$AK81))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M81"/>
       <x:c r="N81"/>
       <x:c r="O81"/>
       <x:c r="P81"/>
@@ -10911,11 +10919,11 @@
       <x:c r="K82" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L82" s="13"/>
-      <x:c r="M82" t="str">
+      <x:c r="L82" s="13" t="str">
         <x:f>IF(TRIM($A82)="","",IF(COUNTIF($Q82:$AK82,"?*")=0,"OK","Falta revisar: "&amp;$Q82&amp;$R82&amp;$S82&amp;$T82&amp;$U82&amp;$V82&amp;$W82&amp;$X82&amp;$Y82&amp;$Z82&amp;$AA82&amp;$AB82&amp;$AC82&amp;$AD82&amp;$AE82&amp;$AF82&amp;$AG82&amp;$AH82&amp;$AI82&amp;$AJ82&amp;$AK82))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M82"/>
       <x:c r="N82"/>
       <x:c r="O82"/>
       <x:c r="P82"/>
@@ -11027,11 +11035,11 @@
       <x:c r="K83" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L83" s="13"/>
-      <x:c r="M83" t="str">
+      <x:c r="L83" s="13" t="str">
         <x:f>IF(TRIM($A83)="","",IF(COUNTIF($Q83:$AK83,"?*")=0,"OK","Falta revisar: "&amp;$Q83&amp;$R83&amp;$S83&amp;$T83&amp;$U83&amp;$V83&amp;$W83&amp;$X83&amp;$Y83&amp;$Z83&amp;$AA83&amp;$AB83&amp;$AC83&amp;$AD83&amp;$AE83&amp;$AF83&amp;$AG83&amp;$AH83&amp;$AI83&amp;$AJ83&amp;$AK83))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M83"/>
       <x:c r="N83"/>
       <x:c r="O83"/>
       <x:c r="P83"/>
@@ -11143,11 +11151,11 @@
       <x:c r="K84" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L84" s="13"/>
-      <x:c r="M84" t="str">
+      <x:c r="L84" s="13" t="str">
         <x:f>IF(TRIM($A84)="","",IF(COUNTIF($Q84:$AK84,"?*")=0,"OK","Falta revisar: "&amp;$Q84&amp;$R84&amp;$S84&amp;$T84&amp;$U84&amp;$V84&amp;$W84&amp;$X84&amp;$Y84&amp;$Z84&amp;$AA84&amp;$AB84&amp;$AC84&amp;$AD84&amp;$AE84&amp;$AF84&amp;$AG84&amp;$AH84&amp;$AI84&amp;$AJ84&amp;$AK84))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M84"/>
       <x:c r="N84"/>
       <x:c r="O84"/>
       <x:c r="P84"/>
@@ -11259,11 +11267,11 @@
       <x:c r="K85" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L85" s="13"/>
-      <x:c r="M85" t="str">
+      <x:c r="L85" s="13" t="str">
         <x:f>IF(TRIM($A85)="","",IF(COUNTIF($Q85:$AK85,"?*")=0,"OK","Falta revisar: "&amp;$Q85&amp;$R85&amp;$S85&amp;$T85&amp;$U85&amp;$V85&amp;$W85&amp;$X85&amp;$Y85&amp;$Z85&amp;$AA85&amp;$AB85&amp;$AC85&amp;$AD85&amp;$AE85&amp;$AF85&amp;$AG85&amp;$AH85&amp;$AI85&amp;$AJ85&amp;$AK85))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M85"/>
       <x:c r="N85"/>
       <x:c r="O85"/>
       <x:c r="P85"/>
@@ -11375,11 +11383,11 @@
       <x:c r="K86" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L86" s="13"/>
-      <x:c r="M86" t="str">
+      <x:c r="L86" s="13" t="str">
         <x:f>IF(TRIM($A86)="","",IF(COUNTIF($Q86:$AK86,"?*")=0,"OK","Falta revisar: "&amp;$Q86&amp;$R86&amp;$S86&amp;$T86&amp;$U86&amp;$V86&amp;$W86&amp;$X86&amp;$Y86&amp;$Z86&amp;$AA86&amp;$AB86&amp;$AC86&amp;$AD86&amp;$AE86&amp;$AF86&amp;$AG86&amp;$AH86&amp;$AI86&amp;$AJ86&amp;$AK86))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M86"/>
       <x:c r="N86"/>
       <x:c r="O86"/>
       <x:c r="P86"/>
@@ -11491,11 +11499,11 @@
       <x:c r="K87" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L87" s="13"/>
-      <x:c r="M87" t="str">
+      <x:c r="L87" s="13" t="str">
         <x:f>IF(TRIM($A87)="","",IF(COUNTIF($Q87:$AK87,"?*")=0,"OK","Falta revisar: "&amp;$Q87&amp;$R87&amp;$S87&amp;$T87&amp;$U87&amp;$V87&amp;$W87&amp;$X87&amp;$Y87&amp;$Z87&amp;$AA87&amp;$AB87&amp;$AC87&amp;$AD87&amp;$AE87&amp;$AF87&amp;$AG87&amp;$AH87&amp;$AI87&amp;$AJ87&amp;$AK87))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M87"/>
       <x:c r="N87"/>
       <x:c r="O87"/>
       <x:c r="P87"/>
@@ -11607,11 +11615,11 @@
       <x:c r="K88" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L88" s="13"/>
-      <x:c r="M88" t="str">
+      <x:c r="L88" s="13" t="str">
         <x:f>IF(TRIM($A88)="","",IF(COUNTIF($Q88:$AK88,"?*")=0,"OK","Falta revisar: "&amp;$Q88&amp;$R88&amp;$S88&amp;$T88&amp;$U88&amp;$V88&amp;$W88&amp;$X88&amp;$Y88&amp;$Z88&amp;$AA88&amp;$AB88&amp;$AC88&amp;$AD88&amp;$AE88&amp;$AF88&amp;$AG88&amp;$AH88&amp;$AI88&amp;$AJ88&amp;$AK88))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M88"/>
       <x:c r="N88"/>
       <x:c r="O88"/>
       <x:c r="P88"/>
@@ -11723,11 +11731,11 @@
       <x:c r="K89" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L89" s="13"/>
-      <x:c r="M89" t="str">
+      <x:c r="L89" s="13" t="str">
         <x:f>IF(TRIM($A89)="","",IF(COUNTIF($Q89:$AK89,"?*")=0,"OK","Falta revisar: "&amp;$Q89&amp;$R89&amp;$S89&amp;$T89&amp;$U89&amp;$V89&amp;$W89&amp;$X89&amp;$Y89&amp;$Z89&amp;$AA89&amp;$AB89&amp;$AC89&amp;$AD89&amp;$AE89&amp;$AF89&amp;$AG89&amp;$AH89&amp;$AI89&amp;$AJ89&amp;$AK89))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M89"/>
       <x:c r="N89"/>
       <x:c r="O89"/>
       <x:c r="P89"/>
@@ -11839,11 +11847,11 @@
       <x:c r="K90" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L90" s="13"/>
-      <x:c r="M90" t="str">
+      <x:c r="L90" s="13" t="str">
         <x:f>IF(TRIM($A90)="","",IF(COUNTIF($Q90:$AK90,"?*")=0,"OK","Falta revisar: "&amp;$Q90&amp;$R90&amp;$S90&amp;$T90&amp;$U90&amp;$V90&amp;$W90&amp;$X90&amp;$Y90&amp;$Z90&amp;$AA90&amp;$AB90&amp;$AC90&amp;$AD90&amp;$AE90&amp;$AF90&amp;$AG90&amp;$AH90&amp;$AI90&amp;$AJ90&amp;$AK90))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M90"/>
       <x:c r="N90"/>
       <x:c r="O90"/>
       <x:c r="P90"/>
@@ -11955,11 +11963,11 @@
       <x:c r="K91" s="11" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L91" s="13"/>
-      <x:c r="M91" t="str">
+      <x:c r="L91" s="13" t="str">
         <x:f>IF(TRIM($A91)="","",IF(COUNTIF($Q91:$AK91,"?*")=0,"OK","Falta revisar: "&amp;$Q91&amp;$R91&amp;$S91&amp;$T91&amp;$U91&amp;$V91&amp;$W91&amp;$X91&amp;$Y91&amp;$Z91&amp;$AA91&amp;$AB91&amp;$AC91&amp;$AD91&amp;$AE91&amp;$AF91&amp;$AG91&amp;$AH91&amp;$AI91&amp;$AJ91&amp;$AK91))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M91"/>
       <x:c r="N91"/>
       <x:c r="O91"/>
       <x:c r="P91"/>
@@ -12071,11 +12079,11 @@
       <x:c r="K92" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L92" s="16"/>
-      <x:c r="M92" t="str">
+      <x:c r="L92" s="16" t="str">
         <x:f>IF(TRIM($A92)="","",IF(COUNTIF($Q92:$AK92,"?*")=0,"OK","Falta revisar: "&amp;$Q92&amp;$R92&amp;$S92&amp;$T92&amp;$U92&amp;$V92&amp;$W92&amp;$X92&amp;$Y92&amp;$Z92&amp;$AA92&amp;$AB92&amp;$AC92&amp;$AD92&amp;$AE92&amp;$AF92&amp;$AG92&amp;$AH92&amp;$AI92&amp;$AJ92&amp;$AK92))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M92"/>
       <x:c r="N92"/>
       <x:c r="O92"/>
       <x:c r="P92"/>
@@ -12187,11 +12195,11 @@
       <x:c r="K93" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L93" s="16"/>
-      <x:c r="M93" t="str">
+      <x:c r="L93" s="16" t="str">
         <x:f>IF(TRIM($A93)="","",IF(COUNTIF($Q93:$AK93,"?*")=0,"OK","Falta revisar: "&amp;$Q93&amp;$R93&amp;$S93&amp;$T93&amp;$U93&amp;$V93&amp;$W93&amp;$X93&amp;$Y93&amp;$Z93&amp;$AA93&amp;$AB93&amp;$AC93&amp;$AD93&amp;$AE93&amp;$AF93&amp;$AG93&amp;$AH93&amp;$AI93&amp;$AJ93&amp;$AK93))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M93"/>
       <x:c r="N93"/>
       <x:c r="O93"/>
       <x:c r="P93"/>
@@ -12303,11 +12311,11 @@
       <x:c r="K94" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L94" s="16"/>
-      <x:c r="M94" t="str">
+      <x:c r="L94" s="16" t="str">
         <x:f>IF(TRIM($A94)="","",IF(COUNTIF($Q94:$AK94,"?*")=0,"OK","Falta revisar: "&amp;$Q94&amp;$R94&amp;$S94&amp;$T94&amp;$U94&amp;$V94&amp;$W94&amp;$X94&amp;$Y94&amp;$Z94&amp;$AA94&amp;$AB94&amp;$AC94&amp;$AD94&amp;$AE94&amp;$AF94&amp;$AG94&amp;$AH94&amp;$AI94&amp;$AJ94&amp;$AK94))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M94"/>
       <x:c r="N94"/>
       <x:c r="O94"/>
       <x:c r="P94"/>
@@ -12419,11 +12427,11 @@
       <x:c r="K95" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L95" s="16"/>
-      <x:c r="M95" t="str">
+      <x:c r="L95" s="16" t="str">
         <x:f>IF(TRIM($A95)="","",IF(COUNTIF($Q95:$AK95,"?*")=0,"OK","Falta revisar: "&amp;$Q95&amp;$R95&amp;$S95&amp;$T95&amp;$U95&amp;$V95&amp;$W95&amp;$X95&amp;$Y95&amp;$Z95&amp;$AA95&amp;$AB95&amp;$AC95&amp;$AD95&amp;$AE95&amp;$AF95&amp;$AG95&amp;$AH95&amp;$AI95&amp;$AJ95&amp;$AK95))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M95"/>
       <x:c r="N95"/>
       <x:c r="O95"/>
       <x:c r="P95"/>
@@ -12535,11 +12543,11 @@
       <x:c r="K96" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L96" s="16"/>
-      <x:c r="M96" t="str">
+      <x:c r="L96" s="16" t="str">
         <x:f>IF(TRIM($A96)="","",IF(COUNTIF($Q96:$AK96,"?*")=0,"OK","Falta revisar: "&amp;$Q96&amp;$R96&amp;$S96&amp;$T96&amp;$U96&amp;$V96&amp;$W96&amp;$X96&amp;$Y96&amp;$Z96&amp;$AA96&amp;$AB96&amp;$AC96&amp;$AD96&amp;$AE96&amp;$AF96&amp;$AG96&amp;$AH96&amp;$AI96&amp;$AJ96&amp;$AK96))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M96"/>
       <x:c r="N96"/>
       <x:c r="O96"/>
       <x:c r="P96"/>
@@ -12651,11 +12659,11 @@
       <x:c r="K97" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L97" s="16"/>
-      <x:c r="M97" t="str">
+      <x:c r="L97" s="16" t="str">
         <x:f>IF(TRIM($A97)="","",IF(COUNTIF($Q97:$AK97,"?*")=0,"OK","Falta revisar: "&amp;$Q97&amp;$R97&amp;$S97&amp;$T97&amp;$U97&amp;$V97&amp;$W97&amp;$X97&amp;$Y97&amp;$Z97&amp;$AA97&amp;$AB97&amp;$AC97&amp;$AD97&amp;$AE97&amp;$AF97&amp;$AG97&amp;$AH97&amp;$AI97&amp;$AJ97&amp;$AK97))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M97"/>
       <x:c r="N97"/>
       <x:c r="O97"/>
       <x:c r="P97"/>
@@ -12767,11 +12775,11 @@
       <x:c r="K98" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L98" s="16"/>
-      <x:c r="M98" t="str">
+      <x:c r="L98" s="16" t="str">
         <x:f>IF(TRIM($A98)="","",IF(COUNTIF($Q98:$AK98,"?*")=0,"OK","Falta revisar: "&amp;$Q98&amp;$R98&amp;$S98&amp;$T98&amp;$U98&amp;$V98&amp;$W98&amp;$X98&amp;$Y98&amp;$Z98&amp;$AA98&amp;$AB98&amp;$AC98&amp;$AD98&amp;$AE98&amp;$AF98&amp;$AG98&amp;$AH98&amp;$AI98&amp;$AJ98&amp;$AK98))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M98"/>
       <x:c r="N98"/>
       <x:c r="O98"/>
       <x:c r="P98"/>
@@ -12883,11 +12891,11 @@
       <x:c r="K99" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L99" s="16"/>
-      <x:c r="M99" t="str">
+      <x:c r="L99" s="16" t="str">
         <x:f>IF(TRIM($A99)="","",IF(COUNTIF($Q99:$AK99,"?*")=0,"OK","Falta revisar: "&amp;$Q99&amp;$R99&amp;$S99&amp;$T99&amp;$U99&amp;$V99&amp;$W99&amp;$X99&amp;$Y99&amp;$Z99&amp;$AA99&amp;$AB99&amp;$AC99&amp;$AD99&amp;$AE99&amp;$AF99&amp;$AG99&amp;$AH99&amp;$AI99&amp;$AJ99&amp;$AK99))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M99"/>
       <x:c r="N99"/>
       <x:c r="O99"/>
       <x:c r="P99"/>
@@ -12999,11 +13007,11 @@
       <x:c r="K100" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L100" s="16"/>
-      <x:c r="M100" t="str">
+      <x:c r="L100" s="16" t="str">
         <x:f>IF(TRIM($A100)="","",IF(COUNTIF($Q100:$AK100,"?*")=0,"OK","Falta revisar: "&amp;$Q100&amp;$R100&amp;$S100&amp;$T100&amp;$U100&amp;$V100&amp;$W100&amp;$X100&amp;$Y100&amp;$Z100&amp;$AA100&amp;$AB100&amp;$AC100&amp;$AD100&amp;$AE100&amp;$AF100&amp;$AG100&amp;$AH100&amp;$AI100&amp;$AJ100&amp;$AK100))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M100"/>
       <x:c r="N100"/>
       <x:c r="O100"/>
       <x:c r="P100"/>
@@ -13115,11 +13123,11 @@
       <x:c r="K101" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L101" s="16"/>
-      <x:c r="M101" t="str">
+      <x:c r="L101" s="16" t="str">
         <x:f>IF(TRIM($A101)="","",IF(COUNTIF($Q101:$AK101,"?*")=0,"OK","Falta revisar: "&amp;$Q101&amp;$R101&amp;$S101&amp;$T101&amp;$U101&amp;$V101&amp;$W101&amp;$X101&amp;$Y101&amp;$Z101&amp;$AA101&amp;$AB101&amp;$AC101&amp;$AD101&amp;$AE101&amp;$AF101&amp;$AG101&amp;$AH101&amp;$AI101&amp;$AJ101&amp;$AK101))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M101"/>
       <x:c r="N101"/>
       <x:c r="O101"/>
       <x:c r="P101"/>
@@ -13231,11 +13239,11 @@
       <x:c r="K102" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L102" s="16"/>
-      <x:c r="M102" t="str">
+      <x:c r="L102" s="16" t="str">
         <x:f>IF(TRIM($A102)="","",IF(COUNTIF($Q102:$AK102,"?*")=0,"OK","Falta revisar: "&amp;$Q102&amp;$R102&amp;$S102&amp;$T102&amp;$U102&amp;$V102&amp;$W102&amp;$X102&amp;$Y102&amp;$Z102&amp;$AA102&amp;$AB102&amp;$AC102&amp;$AD102&amp;$AE102&amp;$AF102&amp;$AG102&amp;$AH102&amp;$AI102&amp;$AJ102&amp;$AK102))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M102"/>
       <x:c r="N102"/>
       <x:c r="O102"/>
       <x:c r="P102"/>
@@ -13347,11 +13355,11 @@
       <x:c r="K103" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L103" s="16"/>
-      <x:c r="M103" t="str">
+      <x:c r="L103" s="16" t="str">
         <x:f>IF(TRIM($A103)="","",IF(COUNTIF($Q103:$AK103,"?*")=0,"OK","Falta revisar: "&amp;$Q103&amp;$R103&amp;$S103&amp;$T103&amp;$U103&amp;$V103&amp;$W103&amp;$X103&amp;$Y103&amp;$Z103&amp;$AA103&amp;$AB103&amp;$AC103&amp;$AD103&amp;$AE103&amp;$AF103&amp;$AG103&amp;$AH103&amp;$AI103&amp;$AJ103&amp;$AK103))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M103"/>
       <x:c r="N103"/>
       <x:c r="O103"/>
       <x:c r="P103"/>
@@ -13463,11 +13471,11 @@
       <x:c r="K104" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L104" s="16"/>
-      <x:c r="M104" t="str">
+      <x:c r="L104" s="16" t="str">
         <x:f>IF(TRIM($A104)="","",IF(COUNTIF($Q104:$AK104,"?*")=0,"OK","Falta revisar: "&amp;$Q104&amp;$R104&amp;$S104&amp;$T104&amp;$U104&amp;$V104&amp;$W104&amp;$X104&amp;$Y104&amp;$Z104&amp;$AA104&amp;$AB104&amp;$AC104&amp;$AD104&amp;$AE104&amp;$AF104&amp;$AG104&amp;$AH104&amp;$AI104&amp;$AJ104&amp;$AK104))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M104"/>
       <x:c r="N104"/>
       <x:c r="O104"/>
       <x:c r="P104"/>
@@ -13579,11 +13587,11 @@
       <x:c r="K105" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L105" s="16"/>
-      <x:c r="M105" t="str">
+      <x:c r="L105" s="16" t="str">
         <x:f>IF(TRIM($A105)="","",IF(COUNTIF($Q105:$AK105,"?*")=0,"OK","Falta revisar: "&amp;$Q105&amp;$R105&amp;$S105&amp;$T105&amp;$U105&amp;$V105&amp;$W105&amp;$X105&amp;$Y105&amp;$Z105&amp;$AA105&amp;$AB105&amp;$AC105&amp;$AD105&amp;$AE105&amp;$AF105&amp;$AG105&amp;$AH105&amp;$AI105&amp;$AJ105&amp;$AK105))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M105"/>
       <x:c r="N105"/>
       <x:c r="O105"/>
       <x:c r="P105"/>
@@ -13695,11 +13703,11 @@
       <x:c r="K106" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L106" s="16"/>
-      <x:c r="M106" t="str">
+      <x:c r="L106" s="16" t="str">
         <x:f>IF(TRIM($A106)="","",IF(COUNTIF($Q106:$AK106,"?*")=0,"OK","Falta revisar: "&amp;$Q106&amp;$R106&amp;$S106&amp;$T106&amp;$U106&amp;$V106&amp;$W106&amp;$X106&amp;$Y106&amp;$Z106&amp;$AA106&amp;$AB106&amp;$AC106&amp;$AD106&amp;$AE106&amp;$AF106&amp;$AG106&amp;$AH106&amp;$AI106&amp;$AJ106&amp;$AK106))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M106"/>
       <x:c r="N106"/>
       <x:c r="O106"/>
       <x:c r="P106"/>
@@ -13811,11 +13819,11 @@
       <x:c r="K107" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L107" s="16"/>
-      <x:c r="M107" t="str">
+      <x:c r="L107" s="16" t="str">
         <x:f>IF(TRIM($A107)="","",IF(COUNTIF($Q107:$AK107,"?*")=0,"OK","Falta revisar: "&amp;$Q107&amp;$R107&amp;$S107&amp;$T107&amp;$U107&amp;$V107&amp;$W107&amp;$X107&amp;$Y107&amp;$Z107&amp;$AA107&amp;$AB107&amp;$AC107&amp;$AD107&amp;$AE107&amp;$AF107&amp;$AG107&amp;$AH107&amp;$AI107&amp;$AJ107&amp;$AK107))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M107"/>
       <x:c r="N107"/>
       <x:c r="O107"/>
       <x:c r="P107"/>
@@ -13927,11 +13935,11 @@
       <x:c r="K108" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L108" s="16"/>
-      <x:c r="M108" t="str">
+      <x:c r="L108" s="16" t="str">
         <x:f>IF(TRIM($A108)="","",IF(COUNTIF($Q108:$AK108,"?*")=0,"OK","Falta revisar: "&amp;$Q108&amp;$R108&amp;$S108&amp;$T108&amp;$U108&amp;$V108&amp;$W108&amp;$X108&amp;$Y108&amp;$Z108&amp;$AA108&amp;$AB108&amp;$AC108&amp;$AD108&amp;$AE108&amp;$AF108&amp;$AG108&amp;$AH108&amp;$AI108&amp;$AJ108&amp;$AK108))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M108"/>
       <x:c r="N108"/>
       <x:c r="O108"/>
       <x:c r="P108"/>
@@ -14043,11 +14051,11 @@
       <x:c r="K109" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L109" s="16"/>
-      <x:c r="M109" t="str">
+      <x:c r="L109" s="16" t="str">
         <x:f>IF(TRIM($A109)="","",IF(COUNTIF($Q109:$AK109,"?*")=0,"OK","Falta revisar: "&amp;$Q109&amp;$R109&amp;$S109&amp;$T109&amp;$U109&amp;$V109&amp;$W109&amp;$X109&amp;$Y109&amp;$Z109&amp;$AA109&amp;$AB109&amp;$AC109&amp;$AD109&amp;$AE109&amp;$AF109&amp;$AG109&amp;$AH109&amp;$AI109&amp;$AJ109&amp;$AK109))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M109"/>
       <x:c r="N109"/>
       <x:c r="O109"/>
       <x:c r="P109"/>
@@ -14159,11 +14167,11 @@
       <x:c r="K110" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L110" s="16"/>
-      <x:c r="M110" t="str">
+      <x:c r="L110" s="16" t="str">
         <x:f>IF(TRIM($A110)="","",IF(COUNTIF($Q110:$AK110,"?*")=0,"OK","Falta revisar: "&amp;$Q110&amp;$R110&amp;$S110&amp;$T110&amp;$U110&amp;$V110&amp;$W110&amp;$X110&amp;$Y110&amp;$Z110&amp;$AA110&amp;$AB110&amp;$AC110&amp;$AD110&amp;$AE110&amp;$AF110&amp;$AG110&amp;$AH110&amp;$AI110&amp;$AJ110&amp;$AK110))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M110"/>
       <x:c r="N110"/>
       <x:c r="O110"/>
       <x:c r="P110"/>
@@ -14275,11 +14283,11 @@
       <x:c r="K111" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L111" s="16"/>
-      <x:c r="M111" t="str">
+      <x:c r="L111" s="16" t="str">
         <x:f>IF(TRIM($A111)="","",IF(COUNTIF($Q111:$AK111,"?*")=0,"OK","Falta revisar: "&amp;$Q111&amp;$R111&amp;$S111&amp;$T111&amp;$U111&amp;$V111&amp;$W111&amp;$X111&amp;$Y111&amp;$Z111&amp;$AA111&amp;$AB111&amp;$AC111&amp;$AD111&amp;$AE111&amp;$AF111&amp;$AG111&amp;$AH111&amp;$AI111&amp;$AJ111&amp;$AK111))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M111"/>
       <x:c r="N111"/>
       <x:c r="O111"/>
       <x:c r="P111"/>
@@ -14391,11 +14399,11 @@
       <x:c r="K112" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L112" s="16"/>
-      <x:c r="M112" t="str">
+      <x:c r="L112" s="16" t="str">
         <x:f>IF(TRIM($A112)="","",IF(COUNTIF($Q112:$AK112,"?*")=0,"OK","Falta revisar: "&amp;$Q112&amp;$R112&amp;$S112&amp;$T112&amp;$U112&amp;$V112&amp;$W112&amp;$X112&amp;$Y112&amp;$Z112&amp;$AA112&amp;$AB112&amp;$AC112&amp;$AD112&amp;$AE112&amp;$AF112&amp;$AG112&amp;$AH112&amp;$AI112&amp;$AJ112&amp;$AK112))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M112"/>
       <x:c r="N112"/>
       <x:c r="O112"/>
       <x:c r="P112"/>
@@ -14507,11 +14515,11 @@
       <x:c r="K113" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L113" s="16"/>
-      <x:c r="M113" t="str">
+      <x:c r="L113" s="16" t="str">
         <x:f>IF(TRIM($A113)="","",IF(COUNTIF($Q113:$AK113,"?*")=0,"OK","Falta revisar: "&amp;$Q113&amp;$R113&amp;$S113&amp;$T113&amp;$U113&amp;$V113&amp;$W113&amp;$X113&amp;$Y113&amp;$Z113&amp;$AA113&amp;$AB113&amp;$AC113&amp;$AD113&amp;$AE113&amp;$AF113&amp;$AG113&amp;$AH113&amp;$AI113&amp;$AJ113&amp;$AK113))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M113"/>
       <x:c r="N113"/>
       <x:c r="O113"/>
       <x:c r="P113"/>
@@ -14623,11 +14631,11 @@
       <x:c r="K114" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L114" s="16"/>
-      <x:c r="M114" t="str">
+      <x:c r="L114" s="16" t="str">
         <x:f>IF(TRIM($A114)="","",IF(COUNTIF($Q114:$AK114,"?*")=0,"OK","Falta revisar: "&amp;$Q114&amp;$R114&amp;$S114&amp;$T114&amp;$U114&amp;$V114&amp;$W114&amp;$X114&amp;$Y114&amp;$Z114&amp;$AA114&amp;$AB114&amp;$AC114&amp;$AD114&amp;$AE114&amp;$AF114&amp;$AG114&amp;$AH114&amp;$AI114&amp;$AJ114&amp;$AK114))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M114"/>
       <x:c r="N114"/>
       <x:c r="O114"/>
       <x:c r="P114"/>
@@ -14739,11 +14747,11 @@
       <x:c r="K115" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L115" s="16"/>
-      <x:c r="M115" t="str">
+      <x:c r="L115" s="16" t="str">
         <x:f>IF(TRIM($A115)="","",IF(COUNTIF($Q115:$AK115,"?*")=0,"OK","Falta revisar: "&amp;$Q115&amp;$R115&amp;$S115&amp;$T115&amp;$U115&amp;$V115&amp;$W115&amp;$X115&amp;$Y115&amp;$Z115&amp;$AA115&amp;$AB115&amp;$AC115&amp;$AD115&amp;$AE115&amp;$AF115&amp;$AG115&amp;$AH115&amp;$AI115&amp;$AJ115&amp;$AK115))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M115"/>
       <x:c r="N115"/>
       <x:c r="O115"/>
       <x:c r="P115"/>
@@ -14855,11 +14863,11 @@
       <x:c r="K116" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L116" s="16"/>
-      <x:c r="M116" t="str">
+      <x:c r="L116" s="16" t="str">
         <x:f>IF(TRIM($A116)="","",IF(COUNTIF($Q116:$AK116,"?*")=0,"OK","Falta revisar: "&amp;$Q116&amp;$R116&amp;$S116&amp;$T116&amp;$U116&amp;$V116&amp;$W116&amp;$X116&amp;$Y116&amp;$Z116&amp;$AA116&amp;$AB116&amp;$AC116&amp;$AD116&amp;$AE116&amp;$AF116&amp;$AG116&amp;$AH116&amp;$AI116&amp;$AJ116&amp;$AK116))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M116"/>
       <x:c r="N116"/>
       <x:c r="O116"/>
       <x:c r="P116"/>
@@ -14971,11 +14979,11 @@
       <x:c r="K117" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L117" s="16"/>
-      <x:c r="M117" t="str">
+      <x:c r="L117" s="16" t="str">
         <x:f>IF(TRIM($A117)="","",IF(COUNTIF($Q117:$AK117,"?*")=0,"OK","Falta revisar: "&amp;$Q117&amp;$R117&amp;$S117&amp;$T117&amp;$U117&amp;$V117&amp;$W117&amp;$X117&amp;$Y117&amp;$Z117&amp;$AA117&amp;$AB117&amp;$AC117&amp;$AD117&amp;$AE117&amp;$AF117&amp;$AG117&amp;$AH117&amp;$AI117&amp;$AJ117&amp;$AK117))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M117"/>
       <x:c r="N117"/>
       <x:c r="O117"/>
       <x:c r="P117"/>
@@ -15087,11 +15095,11 @@
       <x:c r="K118" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L118" s="16"/>
-      <x:c r="M118" t="str">
+      <x:c r="L118" s="16" t="str">
         <x:f>IF(TRIM($A118)="","",IF(COUNTIF($Q118:$AK118,"?*")=0,"OK","Falta revisar: "&amp;$Q118&amp;$R118&amp;$S118&amp;$T118&amp;$U118&amp;$V118&amp;$W118&amp;$X118&amp;$Y118&amp;$Z118&amp;$AA118&amp;$AB118&amp;$AC118&amp;$AD118&amp;$AE118&amp;$AF118&amp;$AG118&amp;$AH118&amp;$AI118&amp;$AJ118&amp;$AK118))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M118"/>
       <x:c r="N118"/>
       <x:c r="O118"/>
       <x:c r="P118"/>
@@ -15203,11 +15211,11 @@
       <x:c r="K119" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L119" s="16"/>
-      <x:c r="M119" t="str">
+      <x:c r="L119" s="16" t="str">
         <x:f>IF(TRIM($A119)="","",IF(COUNTIF($Q119:$AK119,"?*")=0,"OK","Falta revisar: "&amp;$Q119&amp;$R119&amp;$S119&amp;$T119&amp;$U119&amp;$V119&amp;$W119&amp;$X119&amp;$Y119&amp;$Z119&amp;$AA119&amp;$AB119&amp;$AC119&amp;$AD119&amp;$AE119&amp;$AF119&amp;$AG119&amp;$AH119&amp;$AI119&amp;$AJ119&amp;$AK119))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M119"/>
       <x:c r="N119"/>
       <x:c r="O119"/>
       <x:c r="P119"/>
@@ -15319,11 +15327,11 @@
       <x:c r="K120" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L120" s="16"/>
-      <x:c r="M120" t="str">
+      <x:c r="L120" s="16" t="str">
         <x:f>IF(TRIM($A120)="","",IF(COUNTIF($Q120:$AK120,"?*")=0,"OK","Falta revisar: "&amp;$Q120&amp;$R120&amp;$S120&amp;$T120&amp;$U120&amp;$V120&amp;$W120&amp;$X120&amp;$Y120&amp;$Z120&amp;$AA120&amp;$AB120&amp;$AC120&amp;$AD120&amp;$AE120&amp;$AF120&amp;$AG120&amp;$AH120&amp;$AI120&amp;$AJ120&amp;$AK120))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M120"/>
       <x:c r="N120"/>
       <x:c r="O120"/>
       <x:c r="P120"/>
@@ -15435,11 +15443,11 @@
       <x:c r="K121" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L121" s="16"/>
-      <x:c r="M121" t="str">
+      <x:c r="L121" s="16" t="str">
         <x:f>IF(TRIM($A121)="","",IF(COUNTIF($Q121:$AK121,"?*")=0,"OK","Falta revisar: "&amp;$Q121&amp;$R121&amp;$S121&amp;$T121&amp;$U121&amp;$V121&amp;$W121&amp;$X121&amp;$Y121&amp;$Z121&amp;$AA121&amp;$AB121&amp;$AC121&amp;$AD121&amp;$AE121&amp;$AF121&amp;$AG121&amp;$AH121&amp;$AI121&amp;$AJ121&amp;$AK121))</x:f>
         <x:v>OK</x:v>
       </x:c>
+      <x:c r="M121"/>
       <x:c r="N121"/>
       <x:c r="O121"/>
       <x:c r="P121"/>
@@ -15518,11 +15526,12 @@
       </x:c>
     </x:row>
     <x:row r="122" ht="28" customHeight="1">
+      <x:c r="L122"/>
       <x:c r="M122"/>
-      <x:c r="O122" s="39" t="str">
-        <x:v>RESUMEN AUTOMÁTICO · NO EDITAR</x:v>
-      </x:c>
-      <x:c r="P122" s="40"/>
+      <x:c r="O122" s="43" t="str">
+        <x:v>MÍNIMOS DEL 1ER PARCIAL · NO EDITAR</x:v>
+      </x:c>
+      <x:c r="P122" s="44"/>
       <x:c r="Q122"/>
       <x:c r="R122"/>
       <x:c r="S122"/>
@@ -15551,13 +15560,13 @@
     <x:row r="123" ht="20" customHeight="1">
       <x:c r="I123" s="17"/>
       <x:c r="J123"/>
+      <x:c r="L123"/>
       <x:c r="M123"/>
-      <x:c r="O123" s="35" t="str">
-        <x:v>Total Fáciles:</x:v>
-      </x:c>
-      <x:c r="P123" s="41" t="n">
-        <x:f>COUNTIF($J$2:$J$121,1)</x:f>
-        <x:v>30</x:v>
+      <x:c r="O123" s="45" t="str">
+        <x:v>Mínimo Fáciles:</x:v>
+      </x:c>
+      <x:c r="P123" s="46" t="n">
+        <x:v>15</x:v>
       </x:c>
       <x:c r="Q123"/>
       <x:c r="R123"/>
@@ -15587,13 +15596,13 @@
     <x:row r="124" ht="20" customHeight="1">
       <x:c r="I124" s="17"/>
       <x:c r="J124"/>
+      <x:c r="L124"/>
       <x:c r="M124"/>
-      <x:c r="O124" s="35" t="str">
-        <x:v>Total Medias:</x:v>
-      </x:c>
-      <x:c r="P124" s="41" t="n">
-        <x:f>COUNTIF($J$2:$J$121,2)</x:f>
-        <x:v>60</x:v>
+      <x:c r="O124" s="45" t="str">
+        <x:v>Mínimo Medias:</x:v>
+      </x:c>
+      <x:c r="P124" s="46" t="n">
+        <x:v>30</x:v>
       </x:c>
       <x:c r="Q124"/>
       <x:c r="R124"/>
@@ -15623,13 +15632,13 @@
     <x:row r="125" ht="20" customHeight="1">
       <x:c r="I125" s="17"/>
       <x:c r="J125"/>
+      <x:c r="L125"/>
       <x:c r="M125"/>
-      <x:c r="O125" s="37" t="str">
-        <x:v>Total Difíciles:</x:v>
-      </x:c>
-      <x:c r="P125" s="42" t="n">
-        <x:f>COUNTIF($J$2:$J$121,3)</x:f>
-        <x:v>30</x:v>
+      <x:c r="O125" s="47" t="str">
+        <x:v>Mínimo Difíciles:</x:v>
+      </x:c>
+      <x:c r="P125" s="48" t="n">
+        <x:v>15</x:v>
       </x:c>
       <x:c r="Q125"/>
       <x:c r="R125"/>
@@ -15657,6 +15666,7 @@
       <x:c r="AN125"/>
     </x:row>
     <x:row r="126">
+      <x:c r="L126"/>
       <x:c r="M126"/>
       <x:c r="Q126"/>
       <x:c r="R126"/>
@@ -15684,13 +15694,9 @@
       <x:c r="AN126"/>
     </x:row>
     <x:row r="127">
-      <x:c r="I127" s="17" t="s">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="J127" t="n">
-        <x:f>COUNTIF($A$2:$A$121,"Verdadero o Falso Simple")+COUNTIF($A$2:$A$121,"Verdadero o Falso Complejas")+COUNTIF($A$2:$A$121,"Respuesta A/B/Ambas/Ninguna")</x:f>
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="I127" s="17"/>
+      <x:c r="J127"/>
+      <x:c r="L127"/>
       <x:c r="M127"/>
       <x:c r="Q127"/>
       <x:c r="R127"/>
@@ -15718,13 +15724,9 @@
       <x:c r="AN127"/>
     </x:row>
     <x:row r="128">
-      <x:c r="I128" s="17" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="J128" t="n">
-        <x:f>COUNTIF($A$2:$A$121,"Selección de la mejor respuesta")</x:f>
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="I128" s="17"/>
+      <x:c r="J128"/>
+      <x:c r="L128"/>
       <x:c r="M128"/>
       <x:c r="Q128"/>
       <x:c r="R128"/>
@@ -15752,13 +15754,9 @@
       <x:c r="AN128"/>
     </x:row>
     <x:row r="129">
-      <x:c r="I129" s="17" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="J129" t="n">
-        <x:f>COUNTIF($A$2:$A$121,"Subítem de caso o problema")+COUNTIF($A$2:$A$121,"Opción de Emparejamiento Ampliado")</x:f>
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="I129" s="17"/>
+      <x:c r="J129"/>
+      <x:c r="L129"/>
       <x:c r="M129"/>
       <x:c r="Q129"/>
       <x:c r="R129"/>
@@ -15786,6 +15784,7 @@
       <x:c r="AN129"/>
     </x:row>
     <x:row r="130">
+      <x:c r="L130"/>
       <x:c r="M130"/>
       <x:c r="Q130"/>
       <x:c r="R130"/>
@@ -15813,9 +15812,8 @@
       <x:c r="AN130"/>
     </x:row>
     <x:row r="131">
-      <x:c r="A131" s="17" t="s">
-        <x:v>82</x:v>
-      </x:c>
+      <x:c r="A131" s="17"/>
+      <x:c r="L131"/>
       <x:c r="M131"/>
       <x:c r="Q131"/>
       <x:c r="R131"/>
@@ -15843,9 +15841,8 @@
       <x:c r="AN131"/>
     </x:row>
     <x:row r="132">
-      <x:c r="A132" t="s">
-        <x:v>83</x:v>
-      </x:c>
+      <x:c r="A132"/>
+      <x:c r="L132"/>
       <x:c r="M132"/>
       <x:c r="Q132"/>
       <x:c r="R132"/>
@@ -15873,9 +15870,8 @@
       <x:c r="AN132"/>
     </x:row>
     <x:row r="133">
-      <x:c r="A133" t="s">
-        <x:v>84</x:v>
-      </x:c>
+      <x:c r="A133"/>
+      <x:c r="L133"/>
       <x:c r="M133"/>
       <x:c r="Q133"/>
       <x:c r="R133"/>
@@ -15903,9 +15899,8 @@
       <x:c r="AN133"/>
     </x:row>
     <x:row r="134">
-      <x:c r="A134" t="s">
-        <x:v>85</x:v>
-      </x:c>
+      <x:c r="A134"/>
+      <x:c r="L134"/>
       <x:c r="M134"/>
       <x:c r="Q134"/>
       <x:c r="R134"/>
@@ -15933,9 +15928,8 @@
       <x:c r="AN134"/>
     </x:row>
     <x:row r="135">
-      <x:c r="A135" t="s">
-        <x:v>86</x:v>
-      </x:c>
+      <x:c r="A135"/>
+      <x:c r="L135"/>
       <x:c r="M135"/>
       <x:c r="Q135"/>
       <x:c r="R135"/>
@@ -15963,9 +15957,8 @@
       <x:c r="AN135"/>
     </x:row>
     <x:row r="136">
-      <x:c r="A136" t="s">
-        <x:v>87</x:v>
-      </x:c>
+      <x:c r="A136"/>
+      <x:c r="L136"/>
       <x:c r="M136"/>
       <x:c r="Q136"/>
       <x:c r="R136"/>
@@ -15993,9 +15986,8 @@
       <x:c r="AN136"/>
     </x:row>
     <x:row r="137">
-      <x:c r="A137" t="s">
-        <x:v>88</x:v>
-      </x:c>
+      <x:c r="A137"/>
+      <x:c r="L137"/>
       <x:c r="M137"/>
       <x:c r="Q137"/>
       <x:c r="R137"/>
@@ -16023,9 +16015,8 @@
       <x:c r="AN137"/>
     </x:row>
     <x:row r="138">
-      <x:c r="A138" t="s">
-        <x:v>89</x:v>
-      </x:c>
+      <x:c r="A138"/>
+      <x:c r="L138"/>
       <x:c r="M138"/>
       <x:c r="Q138"/>
       <x:c r="R138"/>
@@ -16053,9 +16044,8 @@
       <x:c r="AN138"/>
     </x:row>
     <x:row r="139">
-      <x:c r="A139" t="s">
-        <x:v>90</x:v>
-      </x:c>
+      <x:c r="A139"/>
+      <x:c r="L139"/>
       <x:c r="M139"/>
       <x:c r="Q139"/>
       <x:c r="R139"/>
@@ -16083,9 +16073,8 @@
       <x:c r="AN139"/>
     </x:row>
     <x:row r="140">
-      <x:c r="A140" t="s">
-        <x:v>91</x:v>
-      </x:c>
+      <x:c r="A140"/>
+      <x:c r="L140"/>
       <x:c r="M140"/>
       <x:c r="Q140"/>
       <x:c r="R140"/>
@@ -19097,7 +19086,7 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="L1" s="18" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -19108,13 +19097,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C2" s="6" t="s">
-        <x:v>92</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D2" t="s">
-        <x:v>93</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E2" t="s">
-        <x:v>94</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="F2" t="s">
         <x:v>2</x:v>
@@ -19135,7 +19124,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L2" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -19146,13 +19135,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C3" s="6" t="s">
-        <x:v>96</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D3" t="s">
-        <x:v>93</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E3" t="s">
-        <x:v>94</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="F3" t="s">
         <x:v>2</x:v>
@@ -19173,7 +19162,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L3" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -19184,19 +19173,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="6" t="s">
-        <x:v>97</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D4" t="s">
-        <x:v>98</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="E4" t="s">
-        <x:v>99</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="F4" t="s">
-        <x:v>100</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="G4" t="s">
-        <x:v>101</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="H4" t="s">
         <x:v>2</x:v>
@@ -19211,7 +19200,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L4" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -19222,19 +19211,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>102</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D5" t="s">
-        <x:v>103</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E5" t="s">
-        <x:v>104</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="F5" t="s">
-        <x:v>105</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="G5" t="s">
-        <x:v>106</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="H5" t="s">
         <x:v>2</x:v>
@@ -19249,7 +19238,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L5" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -19260,22 +19249,22 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C6" s="6" t="s">
-        <x:v>107</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="D6" t="s">
-        <x:v>108</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="E6" t="s">
-        <x:v>109</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="F6" t="s">
-        <x:v>110</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="G6" t="s">
-        <x:v>111</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="H6" t="s">
-        <x:v>112</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="I6" t="s">
         <x:v>11</x:v>
@@ -19287,7 +19276,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L6" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -19298,22 +19287,22 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C7" s="6" t="s">
-        <x:v>113</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D7" t="s">
-        <x:v>114</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="E7" t="s">
-        <x:v>115</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="F7" t="s">
-        <x:v>116</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="G7" t="s">
-        <x:v>117</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="H7" t="s">
-        <x:v>118</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="I7" t="s">
         <x:v>17</x:v>
@@ -19325,7 +19314,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L7" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
@@ -19336,19 +19325,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C8" s="6" t="s">
-        <x:v>119</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D8" t="s">
-        <x:v>120</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E8" t="s">
-        <x:v>121</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F8" t="s">
-        <x:v>122</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="G8" t="s">
-        <x:v>123</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="H8" t="s">
         <x:v>2</x:v>
@@ -19363,7 +19352,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L8" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="36" customHeight="1">
@@ -19374,19 +19363,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C9" s="6" t="s">
-        <x:v>124</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="D9" t="s">
-        <x:v>120</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E9" t="s">
-        <x:v>121</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F9" t="s">
-        <x:v>122</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="G9" t="s">
-        <x:v>123</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="H9" t="s">
         <x:v>2</x:v>
@@ -19401,7 +19390,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L9" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -19409,10 +19398,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B10" t="s">
-        <x:v>125</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C10" s="6" t="s">
-        <x:v>126</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="D10" t="s">
         <x:v>2</x:v>
@@ -19439,7 +19428,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L10" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -19447,25 +19436,25 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B11" t="s">
-        <x:v>125</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C11" s="6" t="s">
-        <x:v>127</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="D11" t="s">
-        <x:v>128</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="E11" t="s">
-        <x:v>129</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="F11" t="s">
-        <x:v>130</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="G11" t="s">
-        <x:v>131</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="H11" t="s">
-        <x:v>132</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="I11" t="s">
         <x:v>1</x:v>
@@ -19477,7 +19466,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L11" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -19485,25 +19474,25 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B12" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="D12" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="E12" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F12" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="G12" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="H12" t="s">
         <x:v>125</x:v>
-      </x:c>
-      <x:c r="C12" s="6" t="s">
-        <x:v>133</x:v>
-      </x:c>
-      <x:c r="D12" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="E12" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="F12" t="s">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="G12" t="s">
-        <x:v>137</x:v>
-      </x:c>
-      <x:c r="H12" t="s">
-        <x:v>138</x:v>
       </x:c>
       <x:c r="I12" t="s">
         <x:v>17</x:v>
@@ -19515,7 +19504,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L12" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -19523,16 +19512,16 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B13" t="s">
-        <x:v>139</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C13" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D13" t="s">
-        <x:v>140</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="E13" t="s">
-        <x:v>141</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F13" t="s">
         <x:v>2</x:v>
@@ -19553,7 +19542,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L13" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -19561,10 +19550,10 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B14" t="s">
-        <x:v>139</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C14" s="6" t="s">
-        <x:v>142</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D14" t="s">
         <x:v>2</x:v>
@@ -19591,7 +19580,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L14" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -19599,10 +19588,10 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B15" t="s">
-        <x:v>139</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C15" s="6" t="s">
-        <x:v>143</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D15" t="s">
         <x:v>2</x:v>
@@ -19629,7 +19618,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L15" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -19637,22 +19626,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" t="s">
-        <x:v>144</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="C16" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D16" t="s">
-        <x:v>145</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="E16" t="s">
-        <x:v>146</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="F16" t="s">
-        <x:v>147</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="G16" t="s">
-        <x:v>148</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="H16" t="s">
         <x:v>2</x:v>
@@ -19667,7 +19656,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L16" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -19675,10 +19664,10 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B17" t="s">
-        <x:v>144</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="C17" s="6" t="s">
-        <x:v>149</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D17" t="s">
         <x:v>2</x:v>
@@ -19705,7 +19694,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L17" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -19713,10 +19702,10 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B18" t="s">
-        <x:v>144</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="C18" s="6" t="s">
-        <x:v>150</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="D18" t="s">
         <x:v>2</x:v>
@@ -19743,7 +19732,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="L18" t="s">
-        <x:v>95</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>